<commit_message>
Additional loans: Erick #7 R500 (22 Sep, R500 from 26 Sep), Isaac #8 R500 (22 Sep, R250×2 from 26 Sep); backups
</commit_message>
<xml_diff>
--- a/docs/BW_Payroll_2026-09-19_to_25_AUDITOR.xlsx
+++ b/docs/BW_Payroll_2026-09-19_to_25_AUDITOR.xlsx
@@ -2172,16 +2172,6 @@
         </is>
       </c>
       <c r="U26" s="6"/>
-      <c r="W26" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#10147 Crew pattern — 7 of 9 at a venue, this one says Warehouse: CREW PATTERN: 7 of 9 workers were at a venue on Mon 21 Sep 2026 (FNB Stadium, Fnb stadium) — Erick Mpho Molefe says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
-        </is>
-      </c>
-      <c r="X26" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#10147 STILL OPEN — no decision recorded yet (claimed hours used)</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="0">
@@ -3748,12 +3738,12 @@
       </c>
       <c r="W45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#9979 Manual overlap review: the same employee has another overlapping entry on 2026-09-21 for 07:00-16:00. | #10131 ALREADY PAID — SAME SHIFT AGAIN (duplicate): John was paid Mon 21 Sep 2026 07:00–16:00 · FNB Stadium (Soweto jhb) · Normal · "Strike down" · 9.00 h × R95,00 = R855,00 (payroll 2026-09-19). He now claims 07:00–16:00 · FNB Stadium (Soweto jhb) · Normal · "Strike down" · 9.00 h for the same day. Every hour of this claim is already paid. Nothing is due: R0,00. Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed. System recommended 0.00 h.</t>
+          <t xml:space="preserve">#10131 ALREADY PAID — SAME SHIFT AGAIN (duplicate): John was paid Mon 21 Sep 2026 07:00–16:00 · FNB Stadium (Soweto jhb) · Normal · "Strike down" · 9.00 h × R95,00 = R855,00 (payroll 2026-09-19). He now claims 07:00–16:00 · FNB Stadium (Soweto jhb) · Normal · "Strike down" · 9.00 h for the same day. Every hour of this claim is already paid. Nothing is due: R0,00. Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed. System recommended 0.00 h.</t>
         </is>
       </c>
       <c r="X45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#9979 DECIDED 3.00 h by Bernie Burness 2026-09-23 09:01: ALREADY BILLED Monday 2026-09-21 · 07:00–16:00 · 9.00 h Normal · FNB Stadium · Strike down R855,00 · shift #9857 · in THIS payroll (2026-09-19 → 2026-09-25, not yet paid) | #10131 DECIDED 0.00 h by Bernie Burness 2026-09-23 09:03: Already paid — SAME SHIFT AGAIN (duplicate) — R0,00 still due — approved amount R0,00</t>
+          <t xml:space="preserve">#10131 DECIDED 0.00 h by Bernie Burness 2026-09-23 09:03: Already paid — SAME SHIFT AGAIN (duplicate) — R0,00 still due — approved amount R0,00</t>
         </is>
       </c>
     </row>
@@ -8564,7 +8554,7 @@
         <v>500</v>
       </c>
       <c r="Y7" s="4">
-        <f>MAX(0,500-X7)</f>
+        <f>MAX(0,1000-X7)</f>
       </c>
       <c r="Z7" s="4">
         <f>U7+X7</f>
@@ -8734,7 +8724,7 @@
         <v>1000</v>
       </c>
       <c r="Y9" s="4">
-        <f>MAX(0,1100-X9)</f>
+        <f>MAX(0,1600-X9)</f>
       </c>
       <c r="Z9" s="4">
         <f>U9+X9</f>
@@ -11193,13 +11183,13 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPEN</t>
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
       <c r="B16" s="26">
-        <v>10147</v>
+        <v>10015</v>
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
@@ -11208,22 +11198,22 @@
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-21</t>
+          <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
       <c r="E16" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+          <t xml:space="preserve">07:00–16:00 warehouse</t>
         </is>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Crew pattern — 7 of 9 at a venue, this one says Warehouse</t>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
       <c r="G16" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">CREW PATTERN: 7 of 9 workers were at a venue on Mon 21 Sep 2026 (FNB Stadium, Fnb stadium) — Erick Mpho Molefe says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
         </is>
       </c>
       <c r="H16" s="26"/>
@@ -11231,10 +11221,26 @@
         <v>9</v>
       </c>
       <c r="J16" s="26"/>
-      <c r="K16" s="26"/>
-      <c r="L16" s="26"/>
-      <c r="M16" s="26"/>
-      <c r="N16" s="26"/>
+      <c r="K16" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M16" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 06:40:17</t>
+        </is>
+      </c>
+      <c r="N16" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9800 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="26" t="inlineStr">
@@ -11243,7 +11249,7 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <v>10015</v>
+        <v>10010</v>
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
@@ -11252,109 +11258,109 @@
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-22</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E17" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 warehouse</t>
+          <t xml:space="preserve">07:00–15:00 wharehouse</t>
         </is>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
         </is>
       </c>
       <c r="G17" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: Erick Mpho Molefe worked 07:00–16:00 on 2026-09-24 (Heritage Day) at wharehouse (Normal). Public-holiday work is not paid automatically. Recommended: Venue/event public holiday (Heritage Day): 9 h × R190 (R95 × 2) = R1 710,00. R0 is paid until the owner approves or declines.</t>
         </is>
       </c>
       <c r="H17" s="26"/>
       <c r="I17" s="27">
-        <v>9</v>
-      </c>
-      <c r="J17" s="26"/>
+        <v>8</v>
+      </c>
+      <c r="J17" s="27">
+        <v>7.5</v>
+      </c>
       <c r="K17" s="26" t="inlineStr">
         <is>
+          <t xml:space="preserve">approve adjusted</t>
+        </is>
+      </c>
+      <c r="L17" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M17" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 10:29:03</t>
+        </is>
+      </c>
+      <c r="N17" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B18" s="29">
+        <v>10073</v>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Givemore Chifetete Kuziwa</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="E18" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06:00–18:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F18" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse claimed — but area says “Pretoria and fnb”</t>
+        </is>
+      </c>
+      <c r="G18" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAREHOUSE CLAIMED BUT AREA SAYS “Pretoria and fnb”: Givemore Chifetete Kuziwa selected Warehouse Team at “Warehouse” for 12.00 h on Thu 17 Sep 2026, but wrote the area as “Pretoria and fnb” — that is a venue, not the warehouse. Other workers were at Botanical garden Pretoria that day. If he was at “Pretoria and fnb”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
+        </is>
+      </c>
+      <c r="H18" s="29"/>
+      <c r="I18" s="30">
+        <v>12</v>
+      </c>
+      <c r="J18" s="29"/>
+      <c r="K18" s="29" t="inlineStr">
+        <is>
           <t xml:space="preserve">approve original</t>
         </is>
       </c>
-      <c r="L17" s="26" t="inlineStr">
+      <c r="L18" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M17" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 06:40:17</t>
-        </is>
-      </c>
-      <c r="N17" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9800 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B18" s="26">
-        <v>10010</v>
-      </c>
-      <c r="C18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Erick Mpho Molefe</t>
-        </is>
-      </c>
-      <c r="D18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-24</t>
-        </is>
-      </c>
-      <c r="E18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–15:00 wharehouse</t>
-        </is>
-      </c>
-      <c r="F18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
-        </is>
-      </c>
-      <c r="G18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: Erick Mpho Molefe worked 07:00–16:00 on 2026-09-24 (Heritage Day) at wharehouse (Normal). Public-holiday work is not paid automatically. Recommended: Venue/event public holiday (Heritage Day): 9 h × R190 (R95 × 2) = R1 710,00. R0 is paid until the owner approves or declines.</t>
-        </is>
-      </c>
-      <c r="H18" s="26"/>
-      <c r="I18" s="27">
-        <v>8</v>
-      </c>
-      <c r="J18" s="27">
-        <v>7.5</v>
-      </c>
-      <c r="K18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve adjusted</t>
-        </is>
-      </c>
-      <c r="L18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 10:29:03</t>
-        </is>
-      </c>
-      <c r="N18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
+      <c r="M18" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 08:58:26</t>
+        </is>
+      </c>
+      <c r="N18" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Event/Venue rate chosen — shift #9789 R934,38 → R640,00 (Venue/event: 12 h × R95 → DIFFERENCE ONLY: Paid last week 08:00–16:00 House/Garden 8.00 h × R62,50 = R500,00 (shift #9705, payroll earlier); 06:00–18:00 at a venue = R1 140,00 (R95,00/h); less the House/Garden already paid R500,00; TO PAY THIS WEEK R640,00)</t>
         </is>
       </c>
     </row>
@@ -11365,7 +11371,7 @@
         </is>
       </c>
       <c r="B19" s="29">
-        <v>10073</v>
+        <v>10140</v>
       </c>
       <c r="C19" s="29" t="inlineStr">
         <is>
@@ -11374,29 +11380,31 @@
       </c>
       <c r="D19" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E19" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">06:00–18:00 Warehouse</t>
+          <t xml:space="preserve">08:00–15:00 Garden</t>
         </is>
       </c>
       <c r="F19" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse claimed — but area says “Pretoria and fnb”</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) — Givemore — approved R1 000,00 — CHECK HOURS NEXT WEEK</t>
         </is>
       </c>
       <c r="G19" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">WAREHOUSE CLAIMED BUT AREA SAYS “Pretoria and fnb”: Givemore Chifetete Kuziwa selected Warehouse Team at “Warehouse” for 12.00 h on Thu 17 Sep 2026, but wrote the area as “Pretoria and fnb” — that is a venue, not the warehouse. Other workers were at Botanical garden Pretoria that day. If he was at “Pretoria and fnb”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
+          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day: Givemore (gardener) claimed 08:00–16:00. Owner: double the day = R1 000. VERIFY NEXT WEEK whether he actually worked 8 h or 4 h.</t>
         </is>
       </c>
       <c r="H19" s="29"/>
       <c r="I19" s="30">
-        <v>12</v>
-      </c>
-      <c r="J19" s="29"/>
+        <v>7</v>
+      </c>
+      <c r="J19" s="30">
+        <v>7</v>
+      </c>
       <c r="K19" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">approve original</t>
@@ -11409,74 +11417,72 @@
       </c>
       <c r="M19" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 08:58:26</t>
+          <t xml:space="preserve">2026-09-23 10:31:30</t>
         </is>
       </c>
       <c r="N19" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Event/Venue rate chosen — shift #9789 R934,38 → R640,00 (Venue/event: 12 h × R95 → DIFFERENCE ONLY: Paid last week 08:00–16:00 House/Garden 8.00 h × R62,50 = R500,00 (shift #9705, payroll earlier); 06:00–18:00 at a venue = R1 140,00 (R95,00/h); less the House/Garden already paid R500,00; TO PAY THIS WEEK R640,00)</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — gardener, hours set to 08:00–15:00: 7 h × R62,50 × 2 = R875,00. CHECK NEXT WEEK what time he really worked until.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B20" s="29">
-        <v>10140</v>
-      </c>
-      <c r="C20" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Givemore Chifetete Kuziwa</t>
-        </is>
-      </c>
-      <c r="D20" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-24</t>
-        </is>
-      </c>
-      <c r="E20" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08:00–15:00 Garden</t>
-        </is>
-      </c>
-      <c r="F20" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — Givemore — approved R1 000,00 — CHECK HOURS NEXT WEEK</t>
-        </is>
-      </c>
-      <c r="G20" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day: Givemore (gardener) claimed 08:00–16:00. Owner: double the day = R1 000. VERIFY NEXT WEEK whether he actually worked 8 h or 4 h.</t>
-        </is>
-      </c>
-      <c r="H20" s="29"/>
-      <c r="I20" s="30">
-        <v>7</v>
-      </c>
-      <c r="J20" s="30">
-        <v>7</v>
-      </c>
-      <c r="K20" s="29" t="inlineStr">
+      <c r="B20" s="32">
+        <v>10104</v>
+      </c>
+      <c r="C20" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isaac Mbele</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="E20" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F20" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+        </is>
+      </c>
+      <c r="H20" s="32"/>
+      <c r="I20" s="33">
+        <v>9</v>
+      </c>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">approve original</t>
         </is>
       </c>
-      <c r="L20" s="29" t="inlineStr">
+      <c r="L20" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M20" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 10:31:30</t>
-        </is>
-      </c>
-      <c r="N20" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — gardener, hours set to 08:00–15:00: 7 h × R62,50 × 2 = R875,00. CHECK NEXT WEEK what time he really worked until.</t>
+      <c r="M20" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 08:43:25</t>
+        </is>
+      </c>
+      <c r="N20" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9850 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
@@ -11487,7 +11493,7 @@
         </is>
       </c>
       <c r="B21" s="32">
-        <v>10104</v>
+        <v>10106</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -11496,7 +11502,7 @@
       </c>
       <c r="D21" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-21</t>
+          <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
       <c r="E21" s="32" t="inlineStr">
@@ -11531,12 +11537,12 @@
       </c>
       <c r="M21" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 08:43:25</t>
+          <t xml:space="preserve">2026-09-23 08:43:27</t>
         </is>
       </c>
       <c r="N21" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9850 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9851 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
@@ -11547,7 +11553,7 @@
         </is>
       </c>
       <c r="B22" s="32">
-        <v>10106</v>
+        <v>10118</v>
       </c>
       <c r="C22" s="32" t="inlineStr">
         <is>
@@ -11556,7 +11562,7 @@
       </c>
       <c r="D22" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-22</t>
+          <t xml:space="preserve">2026-09-23</t>
         </is>
       </c>
       <c r="E22" s="32" t="inlineStr">
@@ -11591,12 +11597,12 @@
       </c>
       <c r="M22" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 08:43:27</t>
+          <t xml:space="preserve">2026-09-23 08:43:31</t>
         </is>
       </c>
       <c r="N22" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9851 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9854 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
@@ -11607,7 +11613,7 @@
         </is>
       </c>
       <c r="B23" s="32">
-        <v>10118</v>
+        <v>10125</v>
       </c>
       <c r="C23" s="32" t="inlineStr">
         <is>
@@ -11616,12 +11622,12 @@
       </c>
       <c r="D23" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E23" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+          <t xml:space="preserve">07:00–15:00 Warehouse</t>
         </is>
       </c>
       <c r="F23" s="32" t="inlineStr">
@@ -11636,7 +11642,7 @@
       </c>
       <c r="H23" s="32"/>
       <c r="I23" s="33">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J23" s="32"/>
       <c r="K23" s="32" t="inlineStr">
@@ -11651,12 +11657,12 @@
       </c>
       <c r="M23" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 08:43:31</t>
+          <t xml:space="preserve">2026-09-23 08:43:34</t>
         </is>
       </c>
       <c r="N23" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9854 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9856 R1 620,00 → R0,00 (PUBLIC HOLIDAY — HELD for owner approval — recommended Warehouse public holiday (Heritage Day): 9 h × R162,50 (R81,25 × 2, no meeting deduction) = R1 462,50; R0 until approved)</t>
         </is>
       </c>
     </row>
@@ -11667,7 +11673,7 @@
         </is>
       </c>
       <c r="B24" s="32">
-        <v>10125</v>
+        <v>10141</v>
       </c>
       <c r="C24" s="32" t="inlineStr">
         <is>
@@ -11686,22 +11692,24 @@
       </c>
       <c r="F24" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
         </is>
       </c>
       <c r="G24" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): Isaac Mbele worked 07:00–15:00. Held for owner approval.</t>
         </is>
       </c>
       <c r="H24" s="32"/>
       <c r="I24" s="33">
         <v>8</v>
       </c>
-      <c r="J24" s="32"/>
+      <c r="J24" s="33">
+        <v>7.5</v>
+      </c>
       <c r="K24" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">approve original</t>
+          <t xml:space="preserve">approve adjusted</t>
         </is>
       </c>
       <c r="L24" s="32" t="inlineStr">
@@ -11711,12 +11719,12 @@
       </c>
       <c r="M24" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 08:43:34</t>
+          <t xml:space="preserve">2026-09-23 10:32:01</t>
         </is>
       </c>
       <c r="N24" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9856 R1 620,00 → R0,00 (PUBLIC HOLIDAY — HELD for owner approval — recommended Warehouse public holiday (Heritage Day): 9 h × R162,50 (R81,25 × 2, no meeting deduction) = R1 462,50; R0 until approved)</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
         </is>
       </c>
     </row>
@@ -11727,7 +11735,7 @@
         </is>
       </c>
       <c r="B25" s="32">
-        <v>10141</v>
+        <v>10129</v>
       </c>
       <c r="C25" s="32" t="inlineStr">
         <is>
@@ -11736,34 +11744,32 @@
       </c>
       <c r="D25" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-24</t>
+          <t xml:space="preserve">2026-09-25</t>
         </is>
       </c>
       <c r="E25" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–15:00 Warehouse</t>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
         </is>
       </c>
       <c r="F25" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
       <c r="G25" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): Isaac Mbele worked 07:00–15:00. Held for owner approval.</t>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
         </is>
       </c>
       <c r="H25" s="32"/>
       <c r="I25" s="33">
-        <v>8</v>
-      </c>
-      <c r="J25" s="33">
-        <v>7.5</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="J25" s="32"/>
       <c r="K25" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">approve adjusted</t>
+          <t xml:space="preserve">approve original</t>
         </is>
       </c>
       <c r="L25" s="32" t="inlineStr">
@@ -11773,72 +11779,74 @@
       </c>
       <c r="M25" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 10:32:01</t>
+          <t xml:space="preserve">2026-09-23 08:43:37</t>
         </is>
       </c>
       <c r="N25" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9858 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="32" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B26" s="32">
-        <v>10129</v>
-      </c>
-      <c r="C26" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Isaac Mbele</t>
-        </is>
-      </c>
-      <c r="D26" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-25</t>
-        </is>
-      </c>
-      <c r="E26" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F26" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
-        </is>
-      </c>
-      <c r="G26" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
-        </is>
-      </c>
-      <c r="H26" s="32"/>
-      <c r="I26" s="33">
+      <c r="B26" s="17">
+        <v>10122</v>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">John Simbarashe Mhlanga</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-16</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Botanical gardens event day</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual overlap review</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-16 for 07:00-16:00.</t>
+        </is>
+      </c>
+      <c r="H26" s="17"/>
+      <c r="I26" s="18">
         <v>9</v>
       </c>
-      <c r="J26" s="32"/>
-      <c r="K26" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L26" s="32" t="inlineStr">
+      <c r="J26" s="18">
+        <v>0</v>
+      </c>
+      <c r="K26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">already paid r0</t>
+        </is>
+      </c>
+      <c r="L26" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M26" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 08:43:37</t>
-        </is>
-      </c>
-      <c r="N26" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9858 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+      <c r="M26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 08:53:49</t>
+        </is>
+      </c>
+      <c r="N26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALREADY BILLED Wednesday 2026-09-16 · 07:00–16:00 · 9.00 h Normal · Botanical gardens event day · Running the event at botanical Gardens R750,00 · shift #9766 · PAID in payroll 2026-09-12 → 2026-09-18 (closed)</t>
         </is>
       </c>
     </row>
@@ -11849,7 +11857,7 @@
         </is>
       </c>
       <c r="B27" s="17">
-        <v>10122</v>
+        <v>10132</v>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
@@ -11868,15 +11876,17 @@
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manual overlap review</t>
+          <t xml:space="preserve">ALREADY PAID — WRONG RATE</t>
         </is>
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-16 for 07:00-16:00.</t>
-        </is>
-      </c>
-      <c r="H27" s="17"/>
+          <t xml:space="preserve">John was paid Wed 16 Sep 2026 07:00–16:00 · Botanical gardens event day (Pretoria) · Normal · "Running the event at botanical Gardens" · 9.00 h × R90,00 = R750,00 (payroll 2026-09-12). He now claims 07:00–16:00 · Botanical gardens event day (Pretoria) · Normal · "Running the event at botanical Gardens" · 9.00 h for the same day. Same work type, but the rate paid (R90,00/h) differs from the rule (R95,00/h). • Rate correction on the paid hours 07:00–16:00: 9.00 h — worth R855,00 at the correct rule, R750,00 was paid → +R105,00 Still due: R105,00 (full day 9.00 h at the correct rule = R855,00 − R750,00 already paid). Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
+        </is>
+      </c>
+      <c r="H27" s="18">
+        <v>0</v>
+      </c>
       <c r="I27" s="18">
         <v>9</v>
       </c>
@@ -11885,7 +11895,7 @@
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">already paid r0</t>
+          <t xml:space="preserve">approve adjusted</t>
         </is>
       </c>
       <c r="L27" s="17" t="inlineStr">
@@ -11895,12 +11905,12 @@
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 08:53:49</t>
+          <t xml:space="preserve">2026-09-23 08:56:44</t>
         </is>
       </c>
       <c r="N27" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALREADY BILLED Wednesday 2026-09-16 · 07:00–16:00 · 9.00 h Normal · Botanical gardens event day · Running the event at botanical Gardens R750,00 · shift #9766 · PAID in payroll 2026-09-12 → 2026-09-18 (closed)</t>
+          <t xml:space="preserve">Already paid — WRONG RATE — R105,00 still due — approved amount R105,00</t>
         </is>
       </c>
     </row>
@@ -11911,7 +11921,7 @@
         </is>
       </c>
       <c r="B28" s="17">
-        <v>10132</v>
+        <v>9972</v>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
@@ -11920,32 +11930,30 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-16</t>
+          <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Botanical gardens event day</t>
+          <t xml:space="preserve">15:00–20:00 Music Bus</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALREADY PAID — WRONG RATE</t>
+          <t xml:space="preserve">Manual overlap review</t>
         </is>
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">John was paid Wed 16 Sep 2026 07:00–16:00 · Botanical gardens event day (Pretoria) · Normal · "Running the event at botanical Gardens" · 9.00 h × R90,00 = R750,00 (payroll 2026-09-12). He now claims 07:00–16:00 · Botanical gardens event day (Pretoria) · Normal · "Running the event at botanical Gardens" · 9.00 h for the same day. Same work type, but the rate paid (R90,00/h) differs from the rule (R95,00/h). • Rate correction on the paid hours 07:00–16:00: 9.00 h — worth R855,00 at the correct rule, R750,00 was paid → +R105,00 Still due: R105,00 (full day 9.00 h at the correct rule = R855,00 − R750,00 already paid). Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
-        </is>
-      </c>
-      <c r="H28" s="18">
-        <v>0</v>
-      </c>
+          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-17 for 15:00-20:00.</t>
+        </is>
+      </c>
+      <c r="H28" s="17"/>
       <c r="I28" s="18">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J28" s="18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K28" s="17" t="inlineStr">
         <is>
@@ -11959,12 +11967,12 @@
       </c>
       <c r="M28" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 08:56:44</t>
+          <t xml:space="preserve">2026-09-23 08:56:08</t>
         </is>
       </c>
       <c r="N28" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Already paid — WRONG RATE — R105,00 still due — approved amount R105,00</t>
+          <t xml:space="preserve">ALREADY BILLED Thursday 2026-09-17 · 07:00–16:00 · 9.00 h Normal · FNB Stadium · Setting up R750,00 · shift #9767 · PAID in payroll 2026-09-12 → 2026-09-18 (closed)</t>
         </is>
       </c>
     </row>
@@ -11975,7 +11983,7 @@
         </is>
       </c>
       <c r="B29" s="17">
-        <v>9972</v>
+        <v>10069</v>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
@@ -11994,15 +12002,17 @@
       </c>
       <c r="F29" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manual overlap review</t>
+          <t xml:space="preserve">ALREADY PAID — EXTRA HOURS</t>
         </is>
       </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-17 for 15:00-20:00.</t>
-        </is>
-      </c>
-      <c r="H29" s="17"/>
+          <t xml:space="preserve">John was paid Thu 17 Sep 2026 07:00–16:00 · FNB Stadium (Jhb) · Normal · "Setting up" · 9.00 h × R90,00 = R750,00 (payroll 2026-09-12). He now claims 15:00–20:00 · Music Bus (Thembisa) · Music Bus · "Missed shifts from Thursday doing music bus in Thembisa where there was a trade visit" · 5.00 h for the same day. Work type changed: Normal → Music Bus (rate R90,00 → R120,00). • Extra hours 16:00–20:00: 4.00 h → R480,00 Still due: R480,00 (full day 5.00 h at the correct rule = R1 230,00 − R750,00 already paid). Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
+        </is>
+      </c>
+      <c r="H29" s="18">
+        <v>4</v>
+      </c>
       <c r="I29" s="18">
         <v>5</v>
       </c>
@@ -12021,12 +12031,12 @@
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 08:56:08</t>
+          <t xml:space="preserve">2026-09-23 09:03:50</t>
         </is>
       </c>
       <c r="N29" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALREADY BILLED Thursday 2026-09-17 · 07:00–16:00 · 9.00 h Normal · FNB Stadium · Setting up R750,00 · shift #9767 · PAID in payroll 2026-09-12 → 2026-09-18 (closed)</t>
+          <t xml:space="preserve">Already paid — EXTRA HOURS — R480,00 still due — approved amount R480,00</t>
         </is>
       </c>
     </row>
@@ -12037,7 +12047,7 @@
         </is>
       </c>
       <c r="B30" s="17">
-        <v>10069</v>
+        <v>10072</v>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
@@ -12046,36 +12056,36 @@
       </c>
       <c r="D30" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-21</t>
         </is>
       </c>
       <c r="E30" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">15:00–20:00 Music Bus</t>
+          <t xml:space="preserve">07:00–16:00 FNB Stadium</t>
         </is>
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALREADY PAID — EXTRA HOURS</t>
+          <t xml:space="preserve">ALREADY PAID — SAME SHIFT AGAIN (duplicate)</t>
         </is>
       </c>
       <c r="G30" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">John was paid Thu 17 Sep 2026 07:00–16:00 · FNB Stadium (Jhb) · Normal · "Setting up" · 9.00 h × R90,00 = R750,00 (payroll 2026-09-12). He now claims 15:00–20:00 · Music Bus (Thembisa) · Music Bus · "Missed shifts from Thursday doing music bus in Thembisa where there was a trade visit" · 5.00 h for the same day. Work type changed: Normal → Music Bus (rate R90,00 → R120,00). • Extra hours 16:00–20:00: 4.00 h → R480,00 Still due: R480,00 (full day 5.00 h at the correct rule = R1 230,00 − R750,00 already paid). Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
+          <t xml:space="preserve">John was paid Mon 21 Sep 2026 07:00–16:00 · FNB Stadium (Soweto jhb) · Normal · "Strike down" · 9.00 h × R95,00 = R855,00 (payroll 2026-09-19). He now claims 07:00–16:00 · FNB Stadium (Soweto jhb) · Normal · "Strike down" · 9.00 h for the same day. Every hour of this claim is already paid. Nothing is due: R0,00. Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
         </is>
       </c>
       <c r="H30" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I30" s="18">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J30" s="18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K30" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">approve adjusted</t>
+          <t xml:space="preserve">already paid r0</t>
         </is>
       </c>
       <c r="L30" s="17" t="inlineStr">
@@ -12085,12 +12095,12 @@
       </c>
       <c r="M30" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:03:50</t>
+          <t xml:space="preserve">2026-09-23 09:01:41</t>
         </is>
       </c>
       <c r="N30" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Already paid — EXTRA HOURS — R480,00 still due — approved amount R480,00</t>
+          <t xml:space="preserve">Already paid — SAME SHIFT AGAIN (duplicate) — R0,00 still due — approved amount R0,00</t>
         </is>
       </c>
     </row>
@@ -12101,7 +12111,7 @@
         </is>
       </c>
       <c r="B31" s="17">
-        <v>9979</v>
+        <v>10126</v>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
@@ -12133,11 +12143,11 @@
         <v>9</v>
       </c>
       <c r="J31" s="18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K31" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">approve adjusted</t>
+          <t xml:space="preserve">already paid r0</t>
         </is>
       </c>
       <c r="L31" s="17" t="inlineStr">
@@ -12147,7 +12157,7 @@
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:01:06</t>
+          <t xml:space="preserve">2026-09-23 09:06:06</t>
         </is>
       </c>
       <c r="N31" s="17" t="inlineStr">
@@ -12163,7 +12173,7 @@
         </is>
       </c>
       <c r="B32" s="17">
-        <v>10072</v>
+        <v>10131</v>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
@@ -12211,7 +12221,7 @@
       </c>
       <c r="M32" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:01:41</t>
+          <t xml:space="preserve">2026-09-23 09:03:55</t>
         </is>
       </c>
       <c r="N32" s="17" t="inlineStr">
@@ -12227,7 +12237,7 @@
         </is>
       </c>
       <c r="B33" s="17">
-        <v>10126</v>
+        <v>9983</v>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
@@ -12236,34 +12246,32 @@
       </c>
       <c r="D33" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-21</t>
+          <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
       <c r="E33" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 FNB Stadium</t>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
         </is>
       </c>
       <c r="F33" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manual overlap review</t>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
       <c r="G33" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-21 for 07:00-16:00.</t>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
         </is>
       </c>
       <c r="H33" s="17"/>
       <c r="I33" s="18">
         <v>9</v>
       </c>
-      <c r="J33" s="18">
-        <v>0</v>
-      </c>
+      <c r="J33" s="17"/>
       <c r="K33" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">already paid r0</t>
+          <t xml:space="preserve">approve original</t>
         </is>
       </c>
       <c r="L33" s="17" t="inlineStr">
@@ -12273,12 +12281,12 @@
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:06:06</t>
+          <t xml:space="preserve">2026-09-23 09:02:31</t>
         </is>
       </c>
       <c r="N33" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALREADY BILLED Monday 2026-09-21 · 07:00–16:00 · 9.00 h Normal · FNB Stadium · Strike down R855,00 · shift #9857 · in THIS payroll (2026-09-19 → 2026-09-25, not yet paid)</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9783 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
@@ -12289,7 +12297,7 @@
         </is>
       </c>
       <c r="B34" s="17">
-        <v>10131</v>
+        <v>10092</v>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
@@ -12298,36 +12306,32 @@
       </c>
       <c r="D34" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-21</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E34" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 FNB Stadium</t>
+          <t xml:space="preserve">07:00–12:00 Warehouse</t>
         </is>
       </c>
       <c r="F34" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALREADY PAID — SAME SHIFT AGAIN (duplicate)</t>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
       <c r="G34" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">John was paid Mon 21 Sep 2026 07:00–16:00 · FNB Stadium (Soweto jhb) · Normal · "Strike down" · 9.00 h × R95,00 = R855,00 (payroll 2026-09-19). He now claims 07:00–16:00 · FNB Stadium (Soweto jhb) · Normal · "Strike down" · 9.00 h for the same day. Every hour of this claim is already paid. Nothing is due: R0,00. Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
-        </is>
-      </c>
-      <c r="H34" s="18">
-        <v>0</v>
-      </c>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+        </is>
+      </c>
+      <c r="H34" s="17"/>
       <c r="I34" s="18">
-        <v>9</v>
-      </c>
-      <c r="J34" s="18">
-        <v>0</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="J34" s="17"/>
       <c r="K34" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">already paid r0</t>
+          <t xml:space="preserve">approve original</t>
         </is>
       </c>
       <c r="L34" s="17" t="inlineStr">
@@ -12337,12 +12341,12 @@
       </c>
       <c r="M34" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:03:55</t>
+          <t xml:space="preserve">2026-09-23 09:02:56</t>
         </is>
       </c>
       <c r="N34" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Already paid — SAME SHIFT AGAIN (duplicate) — R0,00 still due — approved amount R0,00</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9846 R900,00 → R0,00 (PUBLIC HOLIDAY — HELD for owner approval — recommended Warehouse public holiday (Heritage Day): 5 h × R162,50 (R81,25 × 2, no meeting deduction) = R812,50; R0 until approved)</t>
         </is>
       </c>
     </row>
@@ -12353,7 +12357,7 @@
         </is>
       </c>
       <c r="B35" s="17">
-        <v>9983</v>
+        <v>10095</v>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
@@ -12362,32 +12366,34 @@
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-22</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+          <t xml:space="preserve">12:00–18:00 Music Bus</t>
         </is>
       </c>
       <c r="F35" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
         </is>
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: John Simbarashe Mhlanga worked 12:00–18:00 on 2026-09-24 (Heritage Day) at Music Bus (Music Bus). Public-holiday work is not paid automatically. Recommended: Music Bus public holiday (Heritage Day): R750 fixed 07–16 + 2 h outside 07–16 × R180 = R1 110,00. R0 is paid until the owner approves or declines.</t>
         </is>
       </c>
       <c r="H35" s="17"/>
       <c r="I35" s="18">
-        <v>9</v>
-      </c>
-      <c r="J35" s="17"/>
+        <v>6</v>
+      </c>
+      <c r="J35" s="18">
+        <v>6</v>
+      </c>
       <c r="K35" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">approve original</t>
+          <t xml:space="preserve">approve adjusted</t>
         </is>
       </c>
       <c r="L35" s="17" t="inlineStr">
@@ -12397,12 +12403,12 @@
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:02:31</t>
+          <t xml:space="preserve">2026-09-23 09:05:05</t>
         </is>
       </c>
       <c r="N35" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9783 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved — R1 110,00 (as recommended)</t>
         </is>
       </c>
     </row>
@@ -12413,7 +12419,7 @@
         </is>
       </c>
       <c r="B36" s="17">
-        <v>10092</v>
+        <v>10144</v>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
@@ -12432,19 +12438,21 @@
       </c>
       <c r="F36" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
         </is>
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): John Simbarashe Mhlanga worked 07:00–12:00. Held for owner approval.</t>
         </is>
       </c>
       <c r="H36" s="17"/>
       <c r="I36" s="18">
         <v>5</v>
       </c>
-      <c r="J36" s="17"/>
+      <c r="J36" s="18">
+        <v>4.5</v>
+      </c>
       <c r="K36" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">approve original</t>
@@ -12457,12 +12465,12 @@
       </c>
       <c r="M36" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:02:56</t>
+          <t xml:space="preserve">2026-09-23 10:31:24</t>
         </is>
       </c>
       <c r="N36" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9846 R900,00 → R0,00 (PUBLIC HOLIDAY — HELD for owner approval — recommended Warehouse public holiday (Heritage Day): 5 h × R162,50 (R81,25 × 2, no meeting deduction) = R812,50; R0 until approved)</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep at the holiday rate: Warehouse public holiday (Heritage Day): 5 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 4.5 h × R162,50 (R81,25 × 2) = R731,25</t>
         </is>
       </c>
     </row>
@@ -12473,7 +12481,7 @@
         </is>
       </c>
       <c r="B37" s="17">
-        <v>10095</v>
+        <v>10098</v>
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
@@ -12482,171 +12490,173 @@
       </c>
       <c r="D37" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-24</t>
+          <t xml:space="preserve">2026-09-25</t>
         </is>
       </c>
       <c r="E37" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">12:00–18:00 Music Bus</t>
+          <t xml:space="preserve">07:00–11:00 Warehouse</t>
         </is>
       </c>
       <c r="F37" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
       <c r="G37" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: John Simbarashe Mhlanga worked 12:00–18:00 on 2026-09-24 (Heritage Day) at Music Bus (Music Bus). Public-holiday work is not paid automatically. Recommended: Music Bus public holiday (Heritage Day): R750 fixed 07–16 + 2 h outside 07–16 × R180 = R1 110,00. R0 is paid until the owner approves or declines.</t>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
         </is>
       </c>
       <c r="H37" s="17"/>
       <c r="I37" s="18">
+        <v>4</v>
+      </c>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L37" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M37" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 09:03:07</t>
+        </is>
+      </c>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9848 R750,00 → R284,38 (Warehouse: 4 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 3.5 h × R81,25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B38" s="20">
+        <v>10109</v>
+      </c>
+      <c r="C38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Joshua Motsamai Nteo</t>
+        </is>
+      </c>
+      <c r="D38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-13</t>
+        </is>
+      </c>
+      <c r="E38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–13:00 Pastdal pretoria</t>
+        </is>
+      </c>
+      <c r="F38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual overlap review</t>
+        </is>
+      </c>
+      <c r="G38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-13 for 07:00-13:00.</t>
+        </is>
+      </c>
+      <c r="H38" s="20"/>
+      <c r="I38" s="21">
         <v>6</v>
       </c>
-      <c r="J37" s="18">
+      <c r="J38" s="21">
+        <v>0</v>
+      </c>
+      <c r="K38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">already paid r0</t>
+        </is>
+      </c>
+      <c r="L38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 09:08:42</t>
+        </is>
+      </c>
+      <c r="N38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALREADY BILLED Sunday 2026-09-13 · 07:00–13:00 · 6.00 h Normal · Pastdal pub · Strikedown R720,00 · shift #9638 · PAID in payroll 2026-09-12 → 2026-09-18 (closed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B39" s="20">
+        <v>10113</v>
+      </c>
+      <c r="C39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Joshua Motsamai Nteo</t>
+        </is>
+      </c>
+      <c r="D39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-13</t>
+        </is>
+      </c>
+      <c r="E39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–13:00 Pastdal pretoria</t>
+        </is>
+      </c>
+      <c r="F39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALREADY PAID — this claim is covered by what was paid</t>
+        </is>
+      </c>
+      <c r="G39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Joshua was paid Sun 13 Sep 2026 07:00–13:00 · Pastdal pub (Pretoria) · Normal · "Strikedown" · 6.00 h × R120,00 = R720,00 (payroll 2026-09-12). He now claims 07:00–13:00 · Pastdal pretoria (Pretoria) · Normal · "Break down" · 6.00 h for the same day. Same work type, but the rate paid (R120,00/h) differs from the rule (R114,00/h). • Rate correction on the paid hours 07:00–13:00: 6.00 h — worth R684,00 at the correct rule, R720,00 was paid → −R36,00 What was paid (R720,00) already covers this claim (R684,00 at the correct rule). Nothing more is due: R0,00. Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
+        </is>
+      </c>
+      <c r="H39" s="21">
+        <v>0</v>
+      </c>
+      <c r="I39" s="21">
         <v>6</v>
       </c>
-      <c r="K37" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve adjusted</t>
-        </is>
-      </c>
-      <c r="L37" s="17" t="inlineStr">
+      <c r="J39" s="21">
+        <v>0</v>
+      </c>
+      <c r="K39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">already paid r0</t>
+        </is>
+      </c>
+      <c r="L39" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M37" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 09:05:05</t>
-        </is>
-      </c>
-      <c r="N37" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved — R1 110,00 (as recommended)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B38" s="17">
-        <v>10144</v>
-      </c>
-      <c r="C38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">John Simbarashe Mhlanga</t>
-        </is>
-      </c>
-      <c r="D38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-24</t>
-        </is>
-      </c>
-      <c r="E38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–12:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
-        </is>
-      </c>
-      <c r="G38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): John Simbarashe Mhlanga worked 07:00–12:00. Held for owner approval.</t>
-        </is>
-      </c>
-      <c r="H38" s="17"/>
-      <c r="I38" s="18">
-        <v>5</v>
-      </c>
-      <c r="J38" s="18">
-        <v>4.5</v>
-      </c>
-      <c r="K38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 10:31:24</t>
-        </is>
-      </c>
-      <c r="N38" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep at the holiday rate: Warehouse public holiday (Heritage Day): 5 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 4.5 h × R162,50 (R81,25 × 2) = R731,25</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B39" s="17">
-        <v>10098</v>
-      </c>
-      <c r="C39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">John Simbarashe Mhlanga</t>
-        </is>
-      </c>
-      <c r="D39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-25</t>
-        </is>
-      </c>
-      <c r="E39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–11:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
-        </is>
-      </c>
-      <c r="G39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
-        </is>
-      </c>
-      <c r="H39" s="17"/>
-      <c r="I39" s="18">
-        <v>4</v>
-      </c>
-      <c r="J39" s="17"/>
-      <c r="K39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 09:03:07</t>
-        </is>
-      </c>
-      <c r="N39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9848 R750,00 → R284,38 (Warehouse: 4 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 3.5 h × R81,25)</t>
+      <c r="M39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 09:21:54</t>
+        </is>
+      </c>
+      <c r="N39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already paid — this claim is covered by what was paid — R0,00 still due — approved amount R0,00</t>
         </is>
       </c>
     </row>
@@ -12657,7 +12667,7 @@
         </is>
       </c>
       <c r="B40" s="20">
-        <v>10109</v>
+        <v>9959</v>
       </c>
       <c r="C40" s="20" t="inlineStr">
         <is>
@@ -12666,34 +12676,32 @@
       </c>
       <c r="D40" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-13</t>
+          <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
       <c r="E40" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–13:00 Pastdal pretoria</t>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
         </is>
       </c>
       <c r="F40" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manual overlap review</t>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
       <c r="G40" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-13 for 07:00-13:00.</t>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
         </is>
       </c>
       <c r="H40" s="20"/>
       <c r="I40" s="21">
-        <v>6</v>
-      </c>
-      <c r="J40" s="21">
-        <v>0</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="J40" s="20"/>
       <c r="K40" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">already paid r0</t>
+          <t xml:space="preserve">approve original</t>
         </is>
       </c>
       <c r="L40" s="20" t="inlineStr">
@@ -12703,12 +12711,12 @@
       </c>
       <c r="M40" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:08:42</t>
+          <t xml:space="preserve">2026-09-23 09:09:09</t>
         </is>
       </c>
       <c r="N40" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALREADY BILLED Sunday 2026-09-13 · 07:00–13:00 · 6.00 h Normal · Pastdal pub · Strikedown R720,00 · shift #9638 · PAID in payroll 2026-09-12 → 2026-09-18 (closed)</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9774 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
@@ -12719,7 +12727,7 @@
         </is>
       </c>
       <c r="B41" s="20">
-        <v>10113</v>
+        <v>9964</v>
       </c>
       <c r="C41" s="20" t="inlineStr">
         <is>
@@ -12728,36 +12736,32 @@
       </c>
       <c r="D41" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-13</t>
+          <t xml:space="preserve">2026-09-23</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–13:00 Pastdal pretoria</t>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
         </is>
       </c>
       <c r="F41" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALREADY PAID — this claim is covered by what was paid</t>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
       <c r="G41" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Joshua was paid Sun 13 Sep 2026 07:00–13:00 · Pastdal pub (Pretoria) · Normal · "Strikedown" · 6.00 h × R120,00 = R720,00 (payroll 2026-09-12). He now claims 07:00–13:00 · Pastdal pretoria (Pretoria) · Normal · "Break down" · 6.00 h for the same day. Same work type, but the rate paid (R120,00/h) differs from the rule (R114,00/h). • Rate correction on the paid hours 07:00–13:00: 6.00 h — worth R684,00 at the correct rule, R720,00 was paid → −R36,00 What was paid (R720,00) already covers this claim (R684,00 at the correct rule). Nothing more is due: R0,00. Hours from Wednesday onwards are estimated for the auditor run; this entry corrects them. Bernie to approve — nothing has been changed.</t>
-        </is>
-      </c>
-      <c r="H41" s="21">
-        <v>0</v>
-      </c>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+        </is>
+      </c>
+      <c r="H41" s="20"/>
       <c r="I41" s="21">
-        <v>6</v>
-      </c>
-      <c r="J41" s="21">
-        <v>0</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="J41" s="20"/>
       <c r="K41" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">already paid r0</t>
+          <t xml:space="preserve">approve original</t>
         </is>
       </c>
       <c r="L41" s="20" t="inlineStr">
@@ -12767,12 +12771,12 @@
       </c>
       <c r="M41" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:21:54</t>
+          <t xml:space="preserve">2026-09-23 09:09:11</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Already paid — this claim is covered by what was paid — R0,00 still due — approved amount R0,00</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9778 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
@@ -12783,7 +12787,7 @@
         </is>
       </c>
       <c r="B42" s="20">
-        <v>9959</v>
+        <v>10110</v>
       </c>
       <c r="C42" s="20" t="inlineStr">
         <is>
@@ -12792,7 +12796,7 @@
       </c>
       <c r="D42" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-22</t>
+          <t xml:space="preserve">2026-09-23</t>
         </is>
       </c>
       <c r="E42" s="20" t="inlineStr">
@@ -12802,22 +12806,24 @@
       </c>
       <c r="F42" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+          <t xml:space="preserve">Manual overlap review</t>
         </is>
       </c>
       <c r="G42" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-23 for 07:00-16:00.</t>
         </is>
       </c>
       <c r="H42" s="20"/>
       <c r="I42" s="21">
         <v>9</v>
       </c>
-      <c r="J42" s="20"/>
+      <c r="J42" s="21">
+        <v>0</v>
+      </c>
       <c r="K42" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">approve original</t>
+          <t xml:space="preserve">already paid r0</t>
         </is>
       </c>
       <c r="L42" s="20" t="inlineStr">
@@ -12827,12 +12833,12 @@
       </c>
       <c r="M42" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:09:09</t>
+          <t xml:space="preserve">2026-09-23 09:20:39</t>
         </is>
       </c>
       <c r="N42" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9774 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+          <t xml:space="preserve">already billed</t>
         </is>
       </c>
     </row>
@@ -12843,7 +12849,7 @@
         </is>
       </c>
       <c r="B43" s="20">
-        <v>9964</v>
+        <v>10111</v>
       </c>
       <c r="C43" s="20" t="inlineStr">
         <is>
@@ -12887,12 +12893,12 @@
       </c>
       <c r="M43" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:09:11</t>
+          <t xml:space="preserve">2026-09-23 09:22:36</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9778 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9853 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
@@ -12903,7 +12909,7 @@
         </is>
       </c>
       <c r="B44" s="20">
-        <v>10110</v>
+        <v>9977</v>
       </c>
       <c r="C44" s="20" t="inlineStr">
         <is>
@@ -12912,34 +12918,32 @@
       </c>
       <c r="D44" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E44" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+          <t xml:space="preserve">07:00–15:00 Warehouse</t>
         </is>
       </c>
       <c r="F44" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manual overlap review</t>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
         </is>
       </c>
       <c r="G44" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same employee has another overlapping entry on 2026-09-23 for 07:00-16:00.</t>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
         </is>
       </c>
       <c r="H44" s="20"/>
       <c r="I44" s="21">
-        <v>9</v>
-      </c>
-      <c r="J44" s="21">
-        <v>0</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="J44" s="20"/>
       <c r="K44" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">already paid r0</t>
+          <t xml:space="preserve">approve original</t>
         </is>
       </c>
       <c r="L44" s="20" t="inlineStr">
@@ -12949,12 +12953,12 @@
       </c>
       <c r="M44" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:20:39</t>
+          <t xml:space="preserve">2026-09-23 09:21:05</t>
         </is>
       </c>
       <c r="N44" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">already billed</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9780 R1 620,00 → R0,00 (PUBLIC HOLIDAY — HELD for owner approval — recommended Warehouse public holiday (Heritage Day): 9 h × R162,50 (R81,25 × 2, no meeting deduction) = R1 462,50; R0 until approved)</t>
         </is>
       </c>
     </row>
@@ -12965,7 +12969,7 @@
         </is>
       </c>
       <c r="B45" s="20">
-        <v>10111</v>
+        <v>10135</v>
       </c>
       <c r="C45" s="20" t="inlineStr">
         <is>
@@ -12974,413 +12978,415 @@
       </c>
       <c r="D45" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+          <t xml:space="preserve">07:00–15:00 Warehouse</t>
         </is>
       </c>
       <c r="F45" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
         </is>
       </c>
       <c r="G45" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): Joshua Motsamai Nteo worked 07:00–16:00 at Warehouse (Meyerton), Cleaning warehouse. Held for owner approval.</t>
         </is>
       </c>
       <c r="H45" s="20"/>
       <c r="I45" s="21">
+        <v>8</v>
+      </c>
+      <c r="J45" s="21">
+        <v>7.5</v>
+      </c>
+      <c r="K45" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve adjusted</t>
+        </is>
+      </c>
+      <c r="L45" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M45" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 10:29:15</t>
+        </is>
+      </c>
+      <c r="N45" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B46" s="23">
+        <v>9954</v>
+      </c>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patrick Ngozo</t>
+        </is>
+      </c>
+      <c r="D46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06:30–16:00 Wearhouse</t>
+        </is>
+      </c>
+      <c r="F46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rate choice: Warehouse or Venue/Event</t>
+        </is>
+      </c>
+      <c r="G46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The wording says Wearhouse — Loading but the work type is Normal. Choose Warehouse (R81,25/h, 9.5 h less 0.5 h staff meeting = R731,25) or Venue/Event (R95/h = R902,50). The shift stays at R795 until you choose.</t>
+        </is>
+      </c>
+      <c r="H46" s="23"/>
+      <c r="I46" s="24">
+        <v>9.5</v>
+      </c>
+      <c r="J46" s="23"/>
+      <c r="K46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22 12:28:15</t>
+        </is>
+      </c>
+      <c r="N46" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9773 R795,00 → R731,25 (Warehouse: 9.5 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 9 h × R81,25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B47" s="23">
+        <v>10143</v>
+      </c>
+      <c r="C47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patrick Ngozo</t>
+        </is>
+      </c>
+      <c r="D47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-24</t>
+        </is>
+      </c>
+      <c r="E47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06:30–15:00 Wearhouse</t>
+        </is>
+      </c>
+      <c r="F47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
+        </is>
+      </c>
+      <c r="G47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): Patrick Ngozo worked 06:30–15:00. Held for owner approval.</t>
+        </is>
+      </c>
+      <c r="H47" s="23"/>
+      <c r="I47" s="24">
+        <v>8.5</v>
+      </c>
+      <c r="J47" s="24">
+        <v>8</v>
+      </c>
+      <c r="K47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 10:30:29</t>
+        </is>
+      </c>
+      <c r="N47" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep at the holiday rate: Warehouse public holiday (Heritage Day), owner set hours 06:30–15:00: 8.5 h − 0.5 h staff meeting = 8 h × R162,50 = R1 300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B48" s="26">
+        <v>10063</v>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solomon Moyo</t>
+        </is>
+      </c>
+      <c r="D48" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="E48" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F48" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+        </is>
+      </c>
+      <c r="G48" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+        </is>
+      </c>
+      <c r="H48" s="26"/>
+      <c r="I48" s="27">
         <v>9</v>
       </c>
-      <c r="J45" s="20"/>
-      <c r="K45" s="20" t="inlineStr">
+      <c r="J48" s="26"/>
+      <c r="K48" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">approve original</t>
         </is>
       </c>
-      <c r="L45" s="20" t="inlineStr">
+      <c r="L48" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M45" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 09:22:36</t>
-        </is>
-      </c>
-      <c r="N45" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9853 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="20" t="inlineStr">
+      <c r="M48" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 10:48:16</t>
+        </is>
+      </c>
+      <c r="N48" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9835 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B46" s="20">
-        <v>9977</v>
-      </c>
-      <c r="C46" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Joshua Motsamai Nteo</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="inlineStr">
+      <c r="B49" s="26">
+        <v>10060</v>
+      </c>
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solomon Moyo</t>
+        </is>
+      </c>
+      <c r="D49" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
-      <c r="E46" s="20" t="inlineStr">
+      <c r="E49" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">07:00–15:00 Warehouse</t>
         </is>
       </c>
-      <c r="F46" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
-        </is>
-      </c>
-      <c r="G46" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
-        </is>
-      </c>
-      <c r="H46" s="20"/>
-      <c r="I46" s="21">
+      <c r="F49" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
+        </is>
+      </c>
+      <c r="G49" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: Solomon Moyo worked 07:00–16:00 on 2026-09-24 (Heritage Day) at Botanical Gardens (Normal). Public-holiday work is not paid automatically. Recommended: Venue/event public holiday (Heritage Day): 9 h × R190 (R95 × 2) = R1 710,00. R0 is paid until the owner approves or declines.</t>
+        </is>
+      </c>
+      <c r="H49" s="26"/>
+      <c r="I49" s="27">
         <v>8</v>
       </c>
-      <c r="J46" s="20"/>
-      <c r="K46" s="20" t="inlineStr">
+      <c r="J49" s="27">
+        <v>7.5</v>
+      </c>
+      <c r="K49" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve adjusted</t>
+        </is>
+      </c>
+      <c r="L49" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bernie Burness</t>
+        </is>
+      </c>
+      <c r="M49" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 10:31:21</t>
+        </is>
+      </c>
+      <c r="N49" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — warehouse, hours set to 07:00–15:00 (worker wrote Botanical Gardens until 16:00): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1 218,75</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESOLVED</t>
+        </is>
+      </c>
+      <c r="B50" s="29">
+        <v>10074</v>
+      </c>
+      <c r="C50" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takavaudza Chokuda</t>
+        </is>
+      </c>
+      <c r="D50" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="E50" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16:00–18:00 FNB</t>
+        </is>
+      </c>
+      <c r="F50" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse claimed — but the entry names “Johannesburg”</t>
+        </is>
+      </c>
+      <c r="G50" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “Johannesburg”: Takavaudza Chokuda selected Warehouse Team at “FNB” for 2.00 h on Thu 17 Sep 2026, but wrote “Johannesburg” — that is a venue, not the warehouse. 6 workers were at a venue that day (Additional 5 hour shift - 17/09/2026 Parys Golf Day, Botanical garden Pretoria, FNB Stadium, Parys golf &amp; country Estate, Parys Country Club, Parys, Botanical gardens, Fnb stadium). If he was at “Johannesburg”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
+        </is>
+      </c>
+      <c r="H50" s="29"/>
+      <c r="I50" s="30">
+        <v>2</v>
+      </c>
+      <c r="J50" s="29"/>
+      <c r="K50" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">approve original</t>
         </is>
       </c>
-      <c r="L46" s="20" t="inlineStr">
+      <c r="L50" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M46" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 09:21:05</t>
-        </is>
-      </c>
-      <c r="N46" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9780 R1 620,00 → R0,00 (PUBLIC HOLIDAY — HELD for owner approval — recommended Warehouse public holiday (Heritage Day): 9 h × R162,50 (R81,25 × 2, no meeting deduction) = R1 462,50; R0 until approved)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="20" t="inlineStr">
+      <c r="M50" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 11:01:57</t>
+        </is>
+      </c>
+      <c r="N50" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Event/Venue rate chosen — shift #9815 R162,50 → R190,00 (Venue/event: 2 h × R95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B47" s="20">
-        <v>10135</v>
-      </c>
-      <c r="C47" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Joshua Motsamai Nteo</t>
-        </is>
-      </c>
-      <c r="D47" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-24</t>
-        </is>
-      </c>
-      <c r="E47" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–15:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F47" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
-        </is>
-      </c>
-      <c r="G47" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): Joshua Motsamai Nteo worked 07:00–16:00 at Warehouse (Meyerton), Cleaning warehouse. Held for owner approval.</t>
-        </is>
-      </c>
-      <c r="H47" s="20"/>
-      <c r="I47" s="21">
-        <v>8</v>
-      </c>
-      <c r="J47" s="21">
-        <v>7.5</v>
-      </c>
-      <c r="K47" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve adjusted</t>
-        </is>
-      </c>
-      <c r="L47" s="20" t="inlineStr">
+      <c r="B51" s="29">
+        <v>9955</v>
+      </c>
+      <c r="C51" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Takavaudza Chokuda</t>
+        </is>
+      </c>
+      <c r="D51" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="E51" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F51" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crew pattern — 8 of 9 at a venue, this one says Warehouse</t>
+        </is>
+      </c>
+      <c r="G51" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CREW PATTERN: 8 of 9 workers were at a venue on Mon 21 Sep 2026 (FNB Stadium, FNB strike down, Fnb stadium) — Takavaudza Chokuda says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
+        </is>
+      </c>
+      <c r="H51" s="29"/>
+      <c r="I51" s="30">
+        <v>9</v>
+      </c>
+      <c r="J51" s="30">
+        <v>9</v>
+      </c>
+      <c r="K51" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L51" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M47" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 10:29:15</t>
-        </is>
-      </c>
-      <c r="N47" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B48" s="23">
-        <v>9954</v>
-      </c>
-      <c r="C48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Patrick Ngozo</t>
-        </is>
-      </c>
-      <c r="D48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-22</t>
-        </is>
-      </c>
-      <c r="E48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06:30–16:00 Wearhouse</t>
-        </is>
-      </c>
-      <c r="F48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Venue/Event</t>
-        </is>
-      </c>
-      <c r="G48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The wording says Wearhouse — Loading but the work type is Normal. Choose Warehouse (R81,25/h, 9.5 h less 0.5 h staff meeting = R731,25) or Venue/Event (R95/h = R902,50). The shift stays at R795 until you choose.</t>
-        </is>
-      </c>
-      <c r="H48" s="23"/>
-      <c r="I48" s="24">
-        <v>9.5</v>
-      </c>
-      <c r="J48" s="23"/>
-      <c r="K48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-22 12:28:15</t>
-        </is>
-      </c>
-      <c r="N48" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9773 R795,00 → R731,25 (Warehouse: 9.5 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 9 h × R81,25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B49" s="23">
-        <v>10143</v>
-      </c>
-      <c r="C49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Patrick Ngozo</t>
-        </is>
-      </c>
-      <c r="D49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-24</t>
-        </is>
-      </c>
-      <c r="E49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06:30–15:00 Wearhouse</t>
-        </is>
-      </c>
-      <c r="F49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
-        </is>
-      </c>
-      <c r="G49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): Patrick Ngozo worked 06:30–15:00. Held for owner approval.</t>
-        </is>
-      </c>
-      <c r="H49" s="23"/>
-      <c r="I49" s="24">
-        <v>8.5</v>
-      </c>
-      <c r="J49" s="24">
-        <v>8</v>
-      </c>
-      <c r="K49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 10:30:29</t>
-        </is>
-      </c>
-      <c r="N49" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep at the holiday rate: Warehouse public holiday (Heritage Day), owner set hours 06:30–15:00: 8.5 h − 0.5 h staff meeting = 8 h × R162,50 = R1 300,00</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B50" s="26">
-        <v>10063</v>
-      </c>
-      <c r="C50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Solomon Moyo</t>
-        </is>
-      </c>
-      <c r="D50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-22</t>
-        </is>
-      </c>
-      <c r="E50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
-        </is>
-      </c>
-      <c r="G50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
-        </is>
-      </c>
-      <c r="H50" s="26"/>
-      <c r="I50" s="27">
-        <v>9</v>
-      </c>
-      <c r="J50" s="26"/>
-      <c r="K50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 10:48:16</t>
-        </is>
-      </c>
-      <c r="N50" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9835 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B51" s="26">
-        <v>10060</v>
-      </c>
-      <c r="C51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Solomon Moyo</t>
-        </is>
-      </c>
-      <c r="D51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-24</t>
-        </is>
-      </c>
-      <c r="E51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–15:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
-        </is>
-      </c>
-      <c r="G51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: Solomon Moyo worked 07:00–16:00 on 2026-09-24 (Heritage Day) at Botanical Gardens (Normal). Public-holiday work is not paid automatically. Recommended: Venue/event public holiday (Heritage Day): 9 h × R190 (R95 × 2) = R1 710,00. R0 is paid until the owner approves or declines.</t>
-        </is>
-      </c>
-      <c r="H51" s="26"/>
-      <c r="I51" s="27">
-        <v>8</v>
-      </c>
-      <c r="J51" s="27">
-        <v>7.5</v>
-      </c>
-      <c r="K51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve adjusted</t>
-        </is>
-      </c>
-      <c r="L51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 10:31:21</t>
-        </is>
-      </c>
-      <c r="N51" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — warehouse, hours set to 07:00–15:00 (worker wrote Botanical Gardens until 16:00): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1 218,75</t>
+      <c r="M51" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 11:01:58</t>
+        </is>
+      </c>
+      <c r="N51" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WAREHOUSE — R81,25/h chosen by Bernie Burness for draft #830 — will pay R690,63 when final-submitted (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
@@ -13391,7 +13397,7 @@
         </is>
       </c>
       <c r="B52" s="29">
-        <v>10074</v>
+        <v>10075</v>
       </c>
       <c r="C52" s="29" t="inlineStr">
         <is>
@@ -13400,27 +13406,27 @@
       </c>
       <c r="D52" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-23</t>
         </is>
       </c>
       <c r="E52" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">16:00–18:00 FNB</t>
+          <t xml:space="preserve">07:00–16:00 Riverside</t>
         </is>
       </c>
       <c r="F52" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse claimed — but the entry names “Johannesburg”</t>
+          <t xml:space="preserve">Warehouse claimed — but the entry names “The vaal”</t>
         </is>
       </c>
       <c r="G52" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “Johannesburg”: Takavaudza Chokuda selected Warehouse Team at “FNB” for 2.00 h on Thu 17 Sep 2026, but wrote “Johannesburg” — that is a venue, not the warehouse. 6 workers were at a venue that day (Additional 5 hour shift - 17/09/2026 Parys Golf Day, Botanical garden Pretoria, FNB Stadium, Parys golf &amp; country Estate, Parys Country Club, Parys, Botanical gardens, Fnb stadium). If he was at “Johannesburg”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
+          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “The vaal”: Takavaudza Chokuda selected Warehouse Team at “Riverside” for 9.00 h on Wed 23 Sep 2026, but wrote “The vaal” — that is a venue, not the warehouse. 6 workers were at a venue that day (Work with the Team, wharehouse, Set up vaal Boating, Riverside sun, Vaal Boating Season, Stone Haven And Riverside Sun). If he was at “The vaal”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
         </is>
       </c>
       <c r="H52" s="29"/>
       <c r="I52" s="30">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J52" s="29"/>
       <c r="K52" s="29" t="inlineStr">
@@ -13440,7 +13446,7 @@
       </c>
       <c r="N52" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Event/Venue rate chosen — shift #9815 R162,50 → R190,00 (Venue/event: 2 h × R95)</t>
+          <t xml:space="preserve">Event/Venue rate chosen — shift #9819 R690,63 → R855,00 (Venue/event: 9 h × R95)</t>
         </is>
       </c>
     </row>
@@ -13451,7 +13457,7 @@
         </is>
       </c>
       <c r="B53" s="29">
-        <v>9955</v>
+        <v>10039</v>
       </c>
       <c r="C53" s="29" t="inlineStr">
         <is>
@@ -13460,34 +13466,34 @@
       </c>
       <c r="D53" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-21</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E53" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+          <t xml:space="preserve">07:00–15:00 Warehouse</t>
         </is>
       </c>
       <c r="F53" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Crew pattern — 8 of 9 at a venue, this one says Warehouse</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
         </is>
       </c>
       <c r="G53" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">CREW PATTERN: 8 of 9 workers were at a venue on Mon 21 Sep 2026 (FNB Stadium, FNB strike down, Fnb stadium) — Takavaudza Chokuda says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
+          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: Takavaudza Chokuda worked 07:00–16:00 on 2026-09-24 (Heritage Day) at Warehouse (Warehouse Team). Public-holiday work is not paid automatically. Recommended: Warehouse public holiday (Heritage Day): 9 h × R162,50 (R81,25 × 2, no meeting deduction) = R1 462,50. R0 is paid until the owner approves or declines.</t>
         </is>
       </c>
       <c r="H53" s="29"/>
       <c r="I53" s="30">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J53" s="30">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="K53" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">approve original</t>
+          <t xml:space="preserve">approve adjusted</t>
         </is>
       </c>
       <c r="L53" s="29" t="inlineStr">
@@ -13497,12 +13503,12 @@
       </c>
       <c r="M53" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 11:01:58</t>
+          <t xml:space="preserve">2026-09-23 10:32:07</t>
         </is>
       </c>
       <c r="N53" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">WAREHOUSE — R81,25/h chosen by Bernie Burness for draft #830 — will pay R690,63 when final-submitted (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
         </is>
       </c>
     </row>
@@ -13513,7 +13519,7 @@
         </is>
       </c>
       <c r="B54" s="29">
-        <v>10075</v>
+        <v>10076</v>
       </c>
       <c r="C54" s="29" t="inlineStr">
         <is>
@@ -13522,22 +13528,22 @@
       </c>
       <c r="D54" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23</t>
+          <t xml:space="preserve">2026-09-25</t>
         </is>
       </c>
       <c r="E54" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Riverside</t>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
         </is>
       </c>
       <c r="F54" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse claimed — but the entry names “The vaal”</t>
+          <t xml:space="preserve">Crew pattern — 7 of 8 at a venue, this one says Warehouse</t>
         </is>
       </c>
       <c r="G54" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">WAREHOUSE CLAIMED BUT THE ENTRY NAMES “The vaal”: Takavaudza Chokuda selected Warehouse Team at “Riverside” for 9.00 h on Wed 23 Sep 2026, but wrote “The vaal” — that is a venue, not the warehouse. 6 workers were at a venue that day (Work with the Team, wharehouse, Set up vaal Boating, Riverside sun, Vaal Boating Season, Stone Haven And Riverside Sun). If he was at “The vaal”, he is due the venue rate (R95/h); if he was really in the warehouse, R81,25/h. Choose below.</t>
+          <t xml:space="preserve">CREW PATTERN: 7 of 8 workers were at a venue on Fri 25 Sep 2026 (The Capital Sandton and Bonitical Emmarentia, Pretoria country club, Botanical, Vaal Boating, Riverside sun, Pretoria Country Club, Capital hotel / botanical gardens JHB) — Takavaudza Chokuda says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
         </is>
       </c>
       <c r="H54" s="29"/>
@@ -13557,134 +13563,132 @@
       </c>
       <c r="M54" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 11:01:57</t>
+          <t xml:space="preserve">2026-09-23 11:01:58</t>
         </is>
       </c>
       <c r="N54" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Event/Venue rate chosen — shift #9819 R690,63 → R855,00 (Venue/event: 9 h × R95)</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9817 R690,63 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="29" t="inlineStr">
+      <c r="A55" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B55" s="29">
-        <v>10039</v>
-      </c>
-      <c r="C55" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Takavaudza Chokuda</t>
-        </is>
-      </c>
-      <c r="D55" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-24</t>
-        </is>
-      </c>
-      <c r="E55" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–15:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F55" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
-        </is>
-      </c>
-      <c r="G55" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: Takavaudza Chokuda worked 07:00–16:00 on 2026-09-24 (Heritage Day) at Warehouse (Warehouse Team). Public-holiday work is not paid automatically. Recommended: Warehouse public holiday (Heritage Day): 9 h × R162,50 (R81,25 × 2, no meeting deduction) = R1 462,50. R0 is paid until the owner approves or declines.</t>
-        </is>
-      </c>
-      <c r="H55" s="29"/>
-      <c r="I55" s="30">
-        <v>8</v>
-      </c>
-      <c r="J55" s="30">
-        <v>7.5</v>
-      </c>
-      <c r="K55" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve adjusted</t>
-        </is>
-      </c>
-      <c r="L55" s="29" t="inlineStr">
+      <c r="B55" s="32">
+        <v>10080</v>
+      </c>
+      <c r="C55" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thandanani Nkala</t>
+        </is>
+      </c>
+      <c r="D55" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-21</t>
+        </is>
+      </c>
+      <c r="E55" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07:00–16:00 FNB Stadium and Warehouse</t>
+        </is>
+      </c>
+      <c r="F55" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+        </is>
+      </c>
+      <c r="G55" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+        </is>
+      </c>
+      <c r="H55" s="32"/>
+      <c r="I55" s="33">
+        <v>9</v>
+      </c>
+      <c r="J55" s="32"/>
+      <c r="K55" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">approve original</t>
+        </is>
+      </c>
+      <c r="L55" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M55" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 10:32:07</t>
-        </is>
-      </c>
-      <c r="N55" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
+      <c r="M55" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 09:24:21</t>
+        </is>
+      </c>
+      <c r="N55" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Event/Venue rate chosen — shift #9840 R750,00 → R855,00 (Venue/event: 9 h × R95)</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="29" t="inlineStr">
+      <c r="A56" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B56" s="29">
-        <v>10076</v>
-      </c>
-      <c r="C56" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Takavaudza Chokuda</t>
-        </is>
-      </c>
-      <c r="D56" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-25</t>
-        </is>
-      </c>
-      <c r="E56" s="29" t="inlineStr">
+      <c r="B56" s="32">
+        <v>10087</v>
+      </c>
+      <c r="C56" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thandanani Nkala</t>
+        </is>
+      </c>
+      <c r="D56" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="E56" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">07:00–16:00 Warehouse</t>
         </is>
       </c>
-      <c r="F56" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Crew pattern — 7 of 8 at a venue, this one says Warehouse</t>
-        </is>
-      </c>
-      <c r="G56" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CREW PATTERN: 7 of 8 workers were at a venue on Fri 25 Sep 2026 (The Capital Sandton and Bonitical Emmarentia, Pretoria country club, Botanical, Vaal Boating, Riverside sun, Pretoria Country Club, Capital hotel / botanical gardens JHB) — Takavaudza Chokuda says Warehouse for 9.00 h. Check he was not at the venue (R95/h would be due).</t>
-        </is>
-      </c>
-      <c r="H56" s="29"/>
-      <c r="I56" s="30">
+      <c r="F56" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+        </is>
+      </c>
+      <c r="G56" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+        </is>
+      </c>
+      <c r="H56" s="32"/>
+      <c r="I56" s="33">
         <v>9</v>
       </c>
-      <c r="J56" s="29"/>
-      <c r="K56" s="29" t="inlineStr">
+      <c r="J56" s="32"/>
+      <c r="K56" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">approve original</t>
         </is>
       </c>
-      <c r="L56" s="29" t="inlineStr">
+      <c r="L56" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M56" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 11:01:58</t>
-        </is>
-      </c>
-      <c r="N56" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9817 R690,63 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+      <c r="M56" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-23 09:24:24</t>
+        </is>
+      </c>
+      <c r="N56" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9844 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
@@ -13695,7 +13699,7 @@
         </is>
       </c>
       <c r="B57" s="32">
-        <v>10080</v>
+        <v>10084</v>
       </c>
       <c r="C57" s="32" t="inlineStr">
         <is>
@@ -13704,12 +13708,12 @@
       </c>
       <c r="D57" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-21</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E57" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 FNB Stadium and Warehouse</t>
+          <t xml:space="preserve">07:00–15:00 Warehouse</t>
         </is>
       </c>
       <c r="F57" s="32" t="inlineStr">
@@ -13724,7 +13728,7 @@
       </c>
       <c r="H57" s="32"/>
       <c r="I57" s="33">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J57" s="32"/>
       <c r="K57" s="32" t="inlineStr">
@@ -13739,12 +13743,12 @@
       </c>
       <c r="M57" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:24:21</t>
+          <t xml:space="preserve">2026-09-23 09:24:33</t>
         </is>
       </c>
       <c r="N57" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Event/Venue rate chosen — shift #9840 R750,00 → R855,00 (Venue/event: 9 h × R95)</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9842 R1 620,00 → R0,00 (PUBLIC HOLIDAY — HELD for owner approval — recommended Warehouse public holiday (Heritage Day): 9 h × R162,50 (R81,25 × 2, no meeting deduction) = R1 462,50; R0 until approved)</t>
         </is>
       </c>
     </row>
@@ -13755,7 +13759,7 @@
         </is>
       </c>
       <c r="B58" s="32">
-        <v>10087</v>
+        <v>10142</v>
       </c>
       <c r="C58" s="32" t="inlineStr">
         <is>
@@ -13764,32 +13768,34 @@
       </c>
       <c r="D58" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-22</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="E58" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
+          <t xml:space="preserve">07:00–15:00 Warehouse</t>
         </is>
       </c>
       <c r="F58" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
         </is>
       </c>
       <c r="G58" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
+          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): Thandanani Nkala worked 07:00–15:00. Held for owner approval.</t>
         </is>
       </c>
       <c r="H58" s="32"/>
       <c r="I58" s="33">
-        <v>9</v>
-      </c>
-      <c r="J58" s="32"/>
+        <v>8</v>
+      </c>
+      <c r="J58" s="33">
+        <v>7.5</v>
+      </c>
       <c r="K58" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">approve original</t>
+          <t xml:space="preserve">approve adjusted</t>
         </is>
       </c>
       <c r="L58" s="32" t="inlineStr">
@@ -13799,12 +13805,12 @@
       </c>
       <c r="M58" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:24:24</t>
+          <t xml:space="preserve">2026-09-23 10:32:12</t>
         </is>
       </c>
       <c r="N58" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9844 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
+          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
         </is>
       </c>
     </row>
@@ -13815,7 +13821,7 @@
         </is>
       </c>
       <c r="B59" s="32">
-        <v>10084</v>
+        <v>10082</v>
       </c>
       <c r="C59" s="32" t="inlineStr">
         <is>
@@ -13824,12 +13830,12 @@
       </c>
       <c r="D59" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-24</t>
+          <t xml:space="preserve">2026-09-25</t>
         </is>
       </c>
       <c r="E59" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">07:00–15:00 Warehouse</t>
+          <t xml:space="preserve">07:00–16:00 Warehouse</t>
         </is>
       </c>
       <c r="F59" s="32" t="inlineStr">
@@ -13844,7 +13850,7 @@
       </c>
       <c r="H59" s="32"/>
       <c r="I59" s="33">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J59" s="32"/>
       <c r="K59" s="32" t="inlineStr">
@@ -13859,194 +13865,72 @@
       </c>
       <c r="M59" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-23 09:24:33</t>
+          <t xml:space="preserve">2026-09-23 09:24:36</t>
         </is>
       </c>
       <c r="N59" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9842 R1 620,00 → R0,00 (PUBLIC HOLIDAY — HELD for owner approval — recommended Warehouse public holiday (Heritage Day): 9 h × R162,50 (R81,25 × 2, no meeting deduction) = R1 462,50; R0 until approved)</t>
+          <t xml:space="preserve">Warehouse rate chosen — shift #9841 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="32" t="inlineStr">
+      <c r="A60" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">RESOLVED</t>
         </is>
       </c>
-      <c r="B60" s="32">
-        <v>10142</v>
-      </c>
-      <c r="C60" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Thandanani Nkala</t>
-        </is>
-      </c>
-      <c r="D60" s="32" t="inlineStr">
+      <c r="B60" s="17">
+        <v>10033</v>
+      </c>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tsotlego Petrus Malakoane</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
-      <c r="E60" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–15:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F60" s="32" t="inlineStr">
+      <c r="E60" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06:30–14:00 Warehouse</t>
+        </is>
+      </c>
+      <c r="F60" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
         </is>
       </c>
-      <c r="G60" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — Heritage Day (24 Sep 2026): Thandanani Nkala worked 07:00–15:00. Held for owner approval.</t>
-        </is>
-      </c>
-      <c r="H60" s="32"/>
-      <c r="I60" s="33">
-        <v>8</v>
-      </c>
-      <c r="J60" s="33">
+      <c r="G60" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: Tsotlego Petrus Malakoane worked 06:30–16:00 on 2026-09-24 (Heritage Day) at Warehouse (Normal). Public-holiday work is not paid automatically. Recommended: Petrus public holiday (Heritage Day): no fixed day — 9.5 h × R160 (R80 × 2) = R1 520,00. R0 is paid until the owner approves or declines.</t>
+        </is>
+      </c>
+      <c r="H60" s="17"/>
+      <c r="I60" s="18">
         <v>7.5</v>
       </c>
-      <c r="K60" s="32" t="inlineStr">
+      <c r="J60" s="18">
+        <v>7</v>
+      </c>
+      <c r="K60" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">approve adjusted</t>
         </is>
       </c>
-      <c r="L60" s="32" t="inlineStr">
+      <c r="L60" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernie Burness</t>
         </is>
       </c>
-      <c r="M60" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 10:32:12</t>
-        </is>
-      </c>
-      <c r="N60" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 07:00–15:00 (no set-ups): Warehouse public holiday (Heritage Day), owner set hours 07:00–15:00: 8.0 h − 0.5 h staff meeting 07:00–07:30 (unpaid) = 7.5 h × R162,50 (R81,25 × 2) = R1218.75</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B61" s="32">
-        <v>10082</v>
-      </c>
-      <c r="C61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Thandanani Nkala</t>
-        </is>
-      </c>
-      <c r="D61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-25</t>
-        </is>
-      </c>
-      <c r="E61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07:00–16:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rate choice: Warehouse or Event/Venue</t>
-        </is>
-      </c>
-      <c r="G61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RATE CHOICE NEEDED: the wording mentions "warehouse" but the work type is Normal, so it is not clearly warehouse-only. Bernie must choose Warehouse (R81,25/h, Sunday R97,50, meeting time unpaid) or Venue/Event (R95/h, Sunday R114) before the rate is decided. Until then the shift stays at the engine amount.</t>
-        </is>
-      </c>
-      <c r="H61" s="32"/>
-      <c r="I61" s="33">
-        <v>9</v>
-      </c>
-      <c r="J61" s="32"/>
-      <c r="K61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve original</t>
-        </is>
-      </c>
-      <c r="L61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-23 09:24:36</t>
-        </is>
-      </c>
-      <c r="N61" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warehouse rate chosen — shift #9841 R750,00 → R690,63 (Warehouse: 9 h − 0.5 h staff meeting 07:00–07:30 (unpaid, R40,63) = 8.5 h × R81,25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RESOLVED</t>
-        </is>
-      </c>
-      <c r="B62" s="17">
-        <v>10033</v>
-      </c>
-      <c r="C62" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tsotlego Petrus Malakoane</t>
-        </is>
-      </c>
-      <c r="D62" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-24</t>
-        </is>
-      </c>
-      <c r="E62" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06:30–14:00 Warehouse</t>
-        </is>
-      </c>
-      <c r="F62" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Public holiday (Heritage Day) — owner to approve or decline</t>
-        </is>
-      </c>
-      <c r="G62" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PUBLIC HOLIDAY — OWNER APPROVAL NEEDED: Tsotlego Petrus Malakoane worked 06:30–16:00 on 2026-09-24 (Heritage Day) at Warehouse (Normal). Public-holiday work is not paid automatically. Recommended: Petrus public holiday (Heritage Day): no fixed day — 9.5 h × R160 (R80 × 2) = R1 520,00. R0 is paid until the owner approves or declines.</t>
-        </is>
-      </c>
-      <c r="H62" s="17"/>
-      <c r="I62" s="18">
-        <v>7.5</v>
-      </c>
-      <c r="J62" s="18">
-        <v>7</v>
-      </c>
-      <c r="K62" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">approve adjusted</t>
-        </is>
-      </c>
-      <c r="L62" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bernie Burness</t>
-        </is>
-      </c>
-      <c r="M62" s="17" t="inlineStr">
+      <c r="M60" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-23 11:02:04</t>
         </is>
       </c>
-      <c r="N62" s="17" t="inlineStr">
+      <c r="N60" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Public holiday (Heritage Day) approved by Bernie Burness 23 Sep — hours set to 06:30–14:00, meeting deducted: 7 h × R160 = R1 120,00. Owner not 100% sure of the end time — CONFIRM NEXT WEEK.</t>
         </is>
@@ -14378,43 +14262,43 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#2</t>
+          <t xml:space="preserve">#7</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Isaac Mbele</t>
+          <t xml:space="preserve">Erick Mpho Molefe</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11</t>
+          <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11</t>
+          <t xml:space="preserve">2026-09-26</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 August Morning mother this week I spent joo aim loan 300 hundred ple</t>
+          <t xml:space="preserve">22 Sep 2026 WhatsApp 07:15: "Goodmorning Mama, can I please have R600 </t>
         </is>
       </c>
       <c r="F13" s="4">
-        <v>900</v>
+        <v>500</v>
       </c>
       <c r="G13" s="4">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="H13" s="4">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="I13" s="5">
-        <v>350</v>
+        <v>500</v>
       </c>
       <c r="J13" s="4">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
@@ -14430,7 +14314,7 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#3</t>
+          <t xml:space="preserve">#2</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
@@ -14440,33 +14324,33 @@
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16</t>
+          <t xml:space="preserve">2026-08-11</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-17</t>
+          <t xml:space="preserve">2026-08-11</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Morning mother joo aim asking 600 hundred loan please</t>
+          <t xml:space="preserve">3 August Morning mother this week I spent joo aim loan 300 hundred ple</t>
         </is>
       </c>
       <c r="F14" s="4">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="G14" s="4">
         <v>250</v>
       </c>
       <c r="H14" s="4">
-        <v>450</v>
+        <v>550</v>
       </c>
       <c r="I14" s="5">
-        <v>150</v>
+        <v>350</v>
       </c>
       <c r="J14" s="4">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
@@ -14482,7 +14366,7 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#6</t>
+          <t xml:space="preserve">#3</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
@@ -14492,175 +14376,201 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-01</t>
+          <t xml:space="preserve">2026-08-16</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-02</t>
+          <t xml:space="preserve">2026-08-17</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Morning mother my kids are having a trip off 1500 but aim short of 600</t>
+          <t xml:space="preserve">Morning mother joo aim asking 600 hundred loan please</t>
         </is>
       </c>
       <c r="F15" s="4">
         <v>600</v>
       </c>
       <c r="G15" s="4">
+        <v>250</v>
+      </c>
+      <c r="H15" s="4">
+        <v>450</v>
+      </c>
+      <c r="I15" s="5">
+        <v>150</v>
+      </c>
+      <c r="J15" s="4">
+        <v>150</v>
+      </c>
+      <c r="K15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weekly</t>
+        </is>
+      </c>
+      <c r="L15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">active</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#6</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isaac Mbele</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-01</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-02</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Morning mother my kids are having a trip off 1500 but aim short of 600</t>
+        </is>
+      </c>
+      <c r="F16" s="4">
         <v>600</v>
       </c>
-      <c r="H15" s="4">
+      <c r="G16" s="4">
+        <v>600</v>
+      </c>
+      <c r="H16" s="4">
         <v>0</v>
       </c>
-      <c r="I15" s="5">
+      <c r="I16" s="5">
         <v>600</v>
       </c>
-      <c r="J15" s="4">
+      <c r="J16" s="4">
         <v>600</v>
       </c>
-      <c r="K15" s="0" t="inlineStr">
+      <c r="K16" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">weekly</t>
         </is>
       </c>
-      <c r="L15" s="0" t="inlineStr">
+      <c r="L16" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">active</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#8</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isaac Mbele</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-26</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22 Sep 2026 WhatsApp 08:15: "Mother so like. Aim not well balanced abo</t>
+        </is>
+      </c>
+      <c r="F17" s="4">
+        <v>500</v>
+      </c>
+      <c r="G17" s="4">
+        <v>250</v>
+      </c>
+      <c r="H17" s="4">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5">
+        <v>500</v>
+      </c>
+      <c r="J17" s="4">
+        <v>0</v>
+      </c>
+      <c r="K17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weekly</t>
+        </is>
+      </c>
+      <c r="L17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">active</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">LOAN REPAYMENT HISTORY (all payrolls)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Loan #</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Employee</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Payroll week</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Recorded at</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Result</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Scheduled</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Deducted</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Balance before</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Balance after</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#1</t>
-        </is>
-      </c>
-      <c r="B19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Erick Mpho Molefe</t>
-        </is>
-      </c>
-      <c r="C19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
-        </is>
-      </c>
-      <c r="D19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-11 10:12</t>
-        </is>
-      </c>
-      <c r="E19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deducted</t>
-        </is>
-      </c>
-      <c r="F19" s="4">
-        <v>500</v>
-      </c>
-      <c r="G19" s="4">
-        <v>500</v>
-      </c>
-      <c r="H19" s="4">
-        <v>2000</v>
-      </c>
-      <c r="I19" s="4">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#1</t>
-        </is>
-      </c>
-      <c r="B20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Erick Mpho Molefe</t>
-        </is>
-      </c>
-      <c r="C20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
-        </is>
-      </c>
-      <c r="D20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-16 13:37</t>
-        </is>
-      </c>
-      <c r="E20" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deducted</t>
-        </is>
-      </c>
-      <c r="F20" s="4">
-        <v>500</v>
-      </c>
-      <c r="G20" s="4">
-        <v>500</v>
-      </c>
-      <c r="H20" s="4">
-        <v>1500</v>
-      </c>
-      <c r="I20" s="4">
-        <v>1000</v>
       </c>
     </row>
     <row r="21">
@@ -14676,12 +14586,12 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07 12:01</t>
+          <t xml:space="preserve">2026-08-11 10:12</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
@@ -14696,70 +14606,70 @@
         <v>500</v>
       </c>
       <c r="H21" s="4">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="I21" s="4">
-        <v>500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#2</t>
+          <t xml:space="preserve">#1</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Isaac Mbele</t>
+          <t xml:space="preserve">Erick Mpho Molefe</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
+          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11 09:42</t>
+          <t xml:space="preserve">2026-08-16 13:37</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">deferred</t>
+          <t xml:space="preserve">deducted</t>
         </is>
       </c>
       <c r="F22" s="4">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G22" s="4">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="H22" s="4">
-        <v>900</v>
+        <v>1500</v>
       </c>
       <c r="I22" s="4">
-        <v>900</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#2</t>
+          <t xml:space="preserve">#1</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Isaac Mbele</t>
+          <t xml:space="preserve">Erick Mpho Molefe</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
+          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16 13:37</t>
+          <t xml:space="preserve">2026-09-07 12:01</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -14768,16 +14678,16 @@
         </is>
       </c>
       <c r="F23" s="4">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G23" s="4">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="H23" s="4">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="I23" s="4">
-        <v>600</v>
+        <v>500</v>
       </c>
     </row>
     <row r="24">
@@ -14793,36 +14703,36 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07 12:01</t>
+          <t xml:space="preserve">2026-08-11 09:42</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">deducted</t>
+          <t xml:space="preserve">deferred</t>
         </is>
       </c>
       <c r="F24" s="4">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="G24" s="4">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="I24" s="4">
-        <v>350</v>
+        <v>900</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#3</t>
+          <t xml:space="preserve">#2</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -14846,22 +14756,22 @@
         </is>
       </c>
       <c r="F25" s="4">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="G25" s="4">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="H25" s="4">
+        <v>900</v>
+      </c>
+      <c r="I25" s="4">
         <v>600</v>
-      </c>
-      <c r="I25" s="4">
-        <v>400</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#3</t>
+          <t xml:space="preserve">#2</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -14891,87 +14801,165 @@
         <v>250</v>
       </c>
       <c r="H26" s="4">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="I26" s="4">
-        <v>150</v>
+        <v>350</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#5</t>
+          <t xml:space="preserve">#3</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Daniel Motaung</t>
+          <t xml:space="preserve">Isaac Mbele</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07 12:01</t>
+          <t xml:space="preserve">2026-08-16 13:37</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">deferred</t>
+          <t xml:space="preserve">deducted</t>
         </is>
       </c>
       <c r="F27" s="4">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="G27" s="4">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H27" s="4">
-        <v>3000</v>
+        <v>600</v>
       </c>
       <c r="I27" s="4">
-        <v>3000</v>
+        <v>400</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">#3</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isaac Mbele</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07 12:01</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deducted</t>
+        </is>
+      </c>
+      <c r="F28" s="4">
+        <v>250</v>
+      </c>
+      <c r="G28" s="4">
+        <v>250</v>
+      </c>
+      <c r="H28" s="4">
+        <v>400</v>
+      </c>
+      <c r="I28" s="4">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#5</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Daniel Motaung</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07 12:01</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deferred</t>
+        </is>
+      </c>
+      <c r="F29" s="4">
+        <v>500</v>
+      </c>
+      <c r="G29" s="4">
+        <v>0</v>
+      </c>
+      <c r="H29" s="4">
+        <v>3000</v>
+      </c>
+      <c r="I29" s="4">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">#6</t>
         </is>
       </c>
-      <c r="B28" s="0" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Isaac Mbele</t>
         </is>
       </c>
-      <c r="C28" s="0" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
         </is>
       </c>
-      <c r="D28" s="0" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-07 12:01</t>
         </is>
       </c>
-      <c r="E28" s="0" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">deferred</t>
         </is>
       </c>
-      <c r="F28" s="4">
+      <c r="F30" s="4">
         <v>600</v>
       </c>
-      <c r="G28" s="4">
+      <c r="G30" s="4">
         <v>0</v>
       </c>
-      <c r="H28" s="4">
+      <c r="H30" s="4">
         <v>600</v>
       </c>
-      <c r="I28" s="4">
+      <c r="I30" s="4">
         <v>600</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Joshua Car Payment fixed deduction R1 000/week from 19 Sep (owner 24 Sep); auditor xlsx refreshed; handover updated
</commit_message>
<xml_diff>
--- a/docs/BW_Payroll_2026-09-19_to_25_AUDITOR.xlsx
+++ b/docs/BW_Payroll_2026-09-19_to_25_AUDITOR.xlsx
@@ -8879,10 +8879,10 @@
         <f>SUM(C11,E11,G11,I11,K11,M11,O11,Q11)</f>
       </c>
       <c r="T11" s="4">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="U11" s="7">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="V11" s="4">
         <f>MAX(0,T11-U11)</f>
@@ -14076,177 +14076,150 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="8">
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Joshua Motsamai Nteo</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Car Payment</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-19</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Car Payments — R1 000 deducted weekly from wages; the accumulated weekly amounts are paid over to Joshua on the 25th of every month (owner instruction Bernie Burness, 24 Sep 2026).</t>
+        </is>
+      </c>
+      <c r="F8" s="4">
+        <v>1000</v>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ongoing</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">ADDITIONAL LOANS</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Loan #</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Employee</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Date given</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Deductions from</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Reason</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Original amount</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Instalment</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Repaid to date</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Outstanding balance</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Due this week</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Frequency</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Status</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Check</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#5</t>
-        </is>
-      </c>
-      <c r="B11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Daniel Motaung</t>
-        </is>
-      </c>
-      <c r="C11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-23</t>
-        </is>
-      </c>
-      <c r="D11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-05</t>
-        </is>
-      </c>
-      <c r="E11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CT SCan Hopital needs money upfront for Scan as medical aid paid the d</t>
-        </is>
-      </c>
-      <c r="F11" s="4">
-        <v>3000</v>
-      </c>
-      <c r="G11" s="4">
-        <v>500</v>
-      </c>
-      <c r="H11" s="4">
-        <v>0</v>
-      </c>
-      <c r="I11" s="5">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4">
-        <v>0</v>
-      </c>
-      <c r="K11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">weekly</t>
-        </is>
-      </c>
-      <c r="L11" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">paid</t>
-        </is>
-      </c>
-      <c r="M11" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Marked PAID but ledger shows only R0,00 repaid of R3 000,00 — please check</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#1</t>
+          <t xml:space="preserve">#5</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erick Mpho Molefe</t>
+          <t xml:space="preserve">Daniel Motaung</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-08</t>
+          <t xml:space="preserve">2026-08-23</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-08</t>
+          <t xml:space="preserve">2026-09-05</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fix car Whatsapp -- send so we need to go check first because we still</t>
+          <t xml:space="preserve">CT SCan Hopital needs money upfront for Scan as medical aid paid the d</t>
         </is>
       </c>
       <c r="F12" s="4">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G12" s="4">
         <v>500</v>
       </c>
       <c r="H12" s="4">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="I12" s="5">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="J12" s="4">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
@@ -14255,14 +14228,19 @@
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">active</t>
+          <t xml:space="preserve">paid</t>
+        </is>
+      </c>
+      <c r="M12" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marked PAID but ledger shows only R0,00 repaid of R3 000,00 — please check</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#7</t>
+          <t xml:space="preserve">#1</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
@@ -14272,33 +14250,33 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-22</t>
+          <t xml:space="preserve">2026-08-08</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-26</t>
+          <t xml:space="preserve">2026-08-08</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">22 Sep 2026 WhatsApp 07:15: "Goodmorning Mama, can I please have R600 </t>
+          <t xml:space="preserve">Fix car Whatsapp -- send so we need to go check first because we still</t>
         </is>
       </c>
       <c r="F13" s="4">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G13" s="4">
         <v>500</v>
       </c>
       <c r="H13" s="4">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="I13" s="5">
         <v>500</v>
       </c>
       <c r="J13" s="4">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
@@ -14314,43 +14292,43 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#2</t>
+          <t xml:space="preserve">#7</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Isaac Mbele</t>
+          <t xml:space="preserve">Erick Mpho Molefe</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11</t>
+          <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11</t>
+          <t xml:space="preserve">2026-09-26</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 August Morning mother this week I spent joo aim loan 300 hundred ple</t>
+          <t xml:space="preserve">22 Sep 2026 WhatsApp 07:15: "Goodmorning Mama, can I please have R600 </t>
         </is>
       </c>
       <c r="F14" s="4">
-        <v>900</v>
+        <v>500</v>
       </c>
       <c r="G14" s="4">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="H14" s="4">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="I14" s="5">
-        <v>350</v>
+        <v>500</v>
       </c>
       <c r="J14" s="4">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
@@ -14366,7 +14344,7 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#3</t>
+          <t xml:space="preserve">#2</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
@@ -14376,33 +14354,33 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16</t>
+          <t xml:space="preserve">2026-08-11</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-17</t>
+          <t xml:space="preserve">2026-08-11</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Morning mother joo aim asking 600 hundred loan please</t>
+          <t xml:space="preserve">3 August Morning mother this week I spent joo aim loan 300 hundred ple</t>
         </is>
       </c>
       <c r="F15" s="4">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="G15" s="4">
         <v>250</v>
       </c>
       <c r="H15" s="4">
-        <v>450</v>
+        <v>550</v>
       </c>
       <c r="I15" s="5">
-        <v>150</v>
+        <v>350</v>
       </c>
       <c r="J15" s="4">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
@@ -14418,7 +14396,7 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#6</t>
+          <t xml:space="preserve">#3</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
@@ -14428,33 +14406,33 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-01</t>
+          <t xml:space="preserve">2026-08-16</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-02</t>
+          <t xml:space="preserve">2026-08-17</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Morning mother my kids are having a trip off 1500 but aim short of 600</t>
+          <t xml:space="preserve">Morning mother joo aim asking 600 hundred loan please</t>
         </is>
       </c>
       <c r="F16" s="4">
         <v>600</v>
       </c>
       <c r="G16" s="4">
-        <v>600</v>
+        <v>250</v>
       </c>
       <c r="H16" s="4">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="I16" s="5">
-        <v>600</v>
+        <v>150</v>
       </c>
       <c r="J16" s="4">
-        <v>600</v>
+        <v>150</v>
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
@@ -14470,7 +14448,7 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#8</t>
+          <t xml:space="preserve">#6</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
@@ -14480,136 +14458,149 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-22</t>
+          <t xml:space="preserve">2026-09-01</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-26</t>
+          <t xml:space="preserve">2026-09-02</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">22 Sep 2026 WhatsApp 08:15: "Mother so like. Aim not well balanced abo</t>
+          <t xml:space="preserve">Morning mother my kids are having a trip off 1500 but aim short of 600</t>
         </is>
       </c>
       <c r="F17" s="4">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="G17" s="4">
-        <v>250</v>
+        <v>600</v>
       </c>
       <c r="H17" s="4">
         <v>0</v>
       </c>
       <c r="I17" s="5">
+        <v>600</v>
+      </c>
+      <c r="J17" s="4">
+        <v>600</v>
+      </c>
+      <c r="K17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weekly</t>
+        </is>
+      </c>
+      <c r="L17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">active</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#8</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isaac Mbele</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-22</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-26</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22 Sep 2026 WhatsApp 08:15: "Mother so like. Aim not well balanced abo</t>
+        </is>
+      </c>
+      <c r="F18" s="4">
         <v>500</v>
       </c>
-      <c r="J17" s="4">
+      <c r="G18" s="4">
+        <v>250</v>
+      </c>
+      <c r="H18" s="4">
         <v>0</v>
       </c>
-      <c r="K17" s="0" t="inlineStr">
+      <c r="I18" s="5">
+        <v>500</v>
+      </c>
+      <c r="J18" s="4">
+        <v>0</v>
+      </c>
+      <c r="K18" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">weekly</t>
         </is>
       </c>
-      <c r="L17" s="0" t="inlineStr">
+      <c r="L18" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">active</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">LOAN REPAYMENT HISTORY (all payrolls)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Loan #</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Employee</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Payroll week</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Recorded at</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Result</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Scheduled</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Deducted</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Balance before</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Balance after</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#1</t>
-        </is>
-      </c>
-      <c r="B21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Erick Mpho Molefe</t>
-        </is>
-      </c>
-      <c r="C21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
-        </is>
-      </c>
-      <c r="D21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-11 10:12</t>
-        </is>
-      </c>
-      <c r="E21" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deducted</t>
-        </is>
-      </c>
-      <c r="F21" s="4">
-        <v>500</v>
-      </c>
-      <c r="G21" s="4">
-        <v>500</v>
-      </c>
-      <c r="H21" s="4">
-        <v>2000</v>
-      </c>
-      <c r="I21" s="4">
-        <v>1500</v>
       </c>
     </row>
     <row r="22">
@@ -14625,12 +14616,12 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
+          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16 13:37</t>
+          <t xml:space="preserve">2026-08-11 10:12</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
@@ -14645,10 +14636,10 @@
         <v>500</v>
       </c>
       <c r="H22" s="4">
+        <v>2000</v>
+      </c>
+      <c r="I22" s="4">
         <v>1500</v>
-      </c>
-      <c r="I22" s="4">
-        <v>1000</v>
       </c>
     </row>
     <row r="23">
@@ -14664,12 +14655,12 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07 12:01</t>
+          <t xml:space="preserve">2026-08-16 13:37</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -14684,49 +14675,49 @@
         <v>500</v>
       </c>
       <c r="H23" s="4">
+        <v>1500</v>
+      </c>
+      <c r="I23" s="4">
         <v>1000</v>
-      </c>
-      <c r="I23" s="4">
-        <v>500</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#2</t>
+          <t xml:space="preserve">#1</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Isaac Mbele</t>
+          <t xml:space="preserve">Erick Mpho Molefe</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
+          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11 09:42</t>
+          <t xml:space="preserve">2026-09-07 12:01</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">deferred</t>
+          <t xml:space="preserve">deducted</t>
         </is>
       </c>
       <c r="F24" s="4">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G24" s="4">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="H24" s="4">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="I24" s="4">
-        <v>900</v>
+        <v>500</v>
       </c>
     </row>
     <row r="25">
@@ -14742,30 +14733,30 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
+          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16 13:37</t>
+          <t xml:space="preserve">2026-08-11 09:42</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">deducted</t>
+          <t xml:space="preserve">deferred</t>
         </is>
       </c>
       <c r="F25" s="4">
         <v>300</v>
       </c>
       <c r="G25" s="4">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H25" s="4">
         <v>900</v>
       </c>
       <c r="I25" s="4">
-        <v>600</v>
+        <v>900</v>
       </c>
     </row>
     <row r="26">
@@ -14781,12 +14772,12 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07 12:01</t>
+          <t xml:space="preserve">2026-08-16 13:37</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -14795,22 +14786,22 @@
         </is>
       </c>
       <c r="F26" s="4">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="G26" s="4">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="H26" s="4">
+        <v>900</v>
+      </c>
+      <c r="I26" s="4">
         <v>600</v>
-      </c>
-      <c r="I26" s="4">
-        <v>350</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#3</t>
+          <t xml:space="preserve">#2</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -14820,12 +14811,12 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
+          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16 13:37</t>
+          <t xml:space="preserve">2026-09-07 12:01</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -14834,16 +14825,16 @@
         </is>
       </c>
       <c r="F27" s="4">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="G27" s="4">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="H27" s="4">
         <v>600</v>
       </c>
       <c r="I27" s="4">
-        <v>400</v>
+        <v>350</v>
       </c>
     </row>
     <row r="28">
@@ -14859,12 +14850,12 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07 12:01</t>
+          <t xml:space="preserve">2026-08-16 13:37</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
@@ -14873,27 +14864,27 @@
         </is>
       </c>
       <c r="F28" s="4">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="G28" s="4">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="H28" s="4">
+        <v>600</v>
+      </c>
+      <c r="I28" s="4">
         <v>400</v>
-      </c>
-      <c r="I28" s="4">
-        <v>150</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#5</t>
+          <t xml:space="preserve">#3</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Daniel Motaung</t>
+          <t xml:space="preserve">Isaac Mbele</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -14908,31 +14899,31 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">deferred</t>
+          <t xml:space="preserve">deducted</t>
         </is>
       </c>
       <c r="F29" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G29" s="4">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="H29" s="4">
-        <v>3000</v>
+        <v>400</v>
       </c>
       <c r="I29" s="4">
-        <v>3000</v>
+        <v>150</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#6</t>
+          <t xml:space="preserve">#5</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Isaac Mbele</t>
+          <t xml:space="preserve">Daniel Motaung</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -14951,15 +14942,54 @@
         </is>
       </c>
       <c r="F30" s="4">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="G30" s="4">
         <v>0</v>
       </c>
       <c r="H30" s="4">
+        <v>3000</v>
+      </c>
+      <c r="I30" s="4">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#6</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isaac Mbele</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07 12:01</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deferred</t>
+        </is>
+      </c>
+      <c r="F31" s="4">
         <v>600</v>
       </c>
-      <c r="I30" s="4">
+      <c r="G31" s="4">
+        <v>0</v>
+      </c>
+      <c r="H31" s="4">
+        <v>600</v>
+      </c>
+      <c r="I31" s="4">
         <v>600</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Joshua Car Payment starts 26 Sep payroll (owner); auditor xlsx 19-25 Sep unchanged from yesterday; handover
</commit_message>
<xml_diff>
--- a/docs/BW_Payroll_2026-09-19_to_25_AUDITOR.xlsx
+++ b/docs/BW_Payroll_2026-09-19_to_25_AUDITOR.xlsx
@@ -8879,10 +8879,10 @@
         <f>SUM(C11,E11,G11,I11,K11,M11,O11,Q11)</f>
       </c>
       <c r="T11" s="4">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="U11" s="7">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="V11" s="4">
         <f>MAX(0,T11-U11)</f>
@@ -14076,150 +14076,177 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Joshua Motsamai Nteo</t>
-        </is>
-      </c>
-      <c r="C8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Car Payment</t>
-        </is>
-      </c>
-      <c r="D8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-19</t>
-        </is>
-      </c>
-      <c r="E8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Car Payments — R1 000 deducted weekly from wages; the accumulated weekly amounts are paid over to Joshua on the 25th of every month (owner instruction Bernie Burness, 24 Sep 2026).</t>
-        </is>
-      </c>
-      <c r="F8" s="4">
-        <v>1000</v>
-      </c>
-      <c r="G8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ongoing</t>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADDITIONAL LOANS</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ADDITIONAL LOANS</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loan #</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Employee</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date given</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deductions from</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reason</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Original amount</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instalment</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repaid to date</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outstanding balance</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Due this week</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frequency</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Loan #</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Employee</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Date given</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Deductions from</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reason</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Original amount</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Instalment</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Repaid to date</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Outstanding balance</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Due this week</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Frequency</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Status</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Check</t>
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#5</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Daniel Motaung</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-23</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-05</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CT SCan Hopital needs money upfront for Scan as medical aid paid the d</t>
+        </is>
+      </c>
+      <c r="F11" s="4">
+        <v>3000</v>
+      </c>
+      <c r="G11" s="4">
+        <v>500</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4">
+        <v>0</v>
+      </c>
+      <c r="K11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">weekly</t>
+        </is>
+      </c>
+      <c r="L11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">paid</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marked PAID but ledger shows only R0,00 repaid of R3 000,00 — please check</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#5</t>
+          <t xml:space="preserve">#1</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Daniel Motaung</t>
+          <t xml:space="preserve">Erick Mpho Molefe</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-23</t>
+          <t xml:space="preserve">2026-08-08</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-05</t>
+          <t xml:space="preserve">2026-08-08</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CT SCan Hopital needs money upfront for Scan as medical aid paid the d</t>
+          <t xml:space="preserve">Fix car Whatsapp -- send so we need to go check first because we still</t>
         </is>
       </c>
       <c r="F12" s="4">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="G12" s="4">
         <v>500</v>
       </c>
       <c r="H12" s="4">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="I12" s="5">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="J12" s="4">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
@@ -14228,19 +14255,14 @@
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">paid</t>
-        </is>
-      </c>
-      <c r="M12" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Marked PAID but ledger shows only R0,00 repaid of R3 000,00 — please check</t>
+          <t xml:space="preserve">active</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#1</t>
+          <t xml:space="preserve">#7</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
@@ -14250,33 +14272,33 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-08</t>
+          <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-08</t>
+          <t xml:space="preserve">2026-09-26</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fix car Whatsapp -- send so we need to go check first because we still</t>
+          <t xml:space="preserve">22 Sep 2026 WhatsApp 07:15: "Goodmorning Mama, can I please have R600 </t>
         </is>
       </c>
       <c r="F13" s="4">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G13" s="4">
         <v>500</v>
       </c>
       <c r="H13" s="4">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="I13" s="5">
         <v>500</v>
       </c>
       <c r="J13" s="4">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="K13" s="0" t="inlineStr">
         <is>
@@ -14292,43 +14314,43 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#7</t>
+          <t xml:space="preserve">#2</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erick Mpho Molefe</t>
+          <t xml:space="preserve">Isaac Mbele</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-22</t>
+          <t xml:space="preserve">2026-08-11</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-26</t>
+          <t xml:space="preserve">2026-08-11</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">22 Sep 2026 WhatsApp 07:15: "Goodmorning Mama, can I please have R600 </t>
+          <t xml:space="preserve">3 August Morning mother this week I spent joo aim loan 300 hundred ple</t>
         </is>
       </c>
       <c r="F14" s="4">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="G14" s="4">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H14" s="4">
-        <v>0</v>
+        <v>550</v>
       </c>
       <c r="I14" s="5">
-        <v>500</v>
+        <v>350</v>
       </c>
       <c r="J14" s="4">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
@@ -14344,7 +14366,7 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#2</t>
+          <t xml:space="preserve">#3</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
@@ -14354,33 +14376,33 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11</t>
+          <t xml:space="preserve">2026-08-16</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11</t>
+          <t xml:space="preserve">2026-08-17</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 August Morning mother this week I spent joo aim loan 300 hundred ple</t>
+          <t xml:space="preserve">Morning mother joo aim asking 600 hundred loan please</t>
         </is>
       </c>
       <c r="F15" s="4">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4">
         <v>250</v>
       </c>
       <c r="H15" s="4">
-        <v>550</v>
+        <v>450</v>
       </c>
       <c r="I15" s="5">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="J15" s="4">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
@@ -14396,7 +14418,7 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#3</t>
+          <t xml:space="preserve">#6</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
@@ -14406,33 +14428,33 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16</t>
+          <t xml:space="preserve">2026-09-01</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-17</t>
+          <t xml:space="preserve">2026-09-02</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Morning mother joo aim asking 600 hundred loan please</t>
+          <t xml:space="preserve">Morning mother my kids are having a trip off 1500 but aim short of 600</t>
         </is>
       </c>
       <c r="F16" s="4">
         <v>600</v>
       </c>
       <c r="G16" s="4">
-        <v>250</v>
+        <v>600</v>
       </c>
       <c r="H16" s="4">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="I16" s="5">
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="J16" s="4">
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
@@ -14448,7 +14470,7 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#6</t>
+          <t xml:space="preserve">#8</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
@@ -14458,33 +14480,33 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-01</t>
+          <t xml:space="preserve">2026-09-22</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-02</t>
+          <t xml:space="preserve">2026-09-26</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Morning mother my kids are having a trip off 1500 but aim short of 600</t>
+          <t xml:space="preserve">22 Sep 2026 WhatsApp 08:15: "Mother so like. Aim not well balanced abo</t>
         </is>
       </c>
       <c r="F17" s="4">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="G17" s="4">
-        <v>600</v>
+        <v>250</v>
       </c>
       <c r="H17" s="4">
         <v>0</v>
       </c>
       <c r="I17" s="5">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="J17" s="4">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
@@ -14497,110 +14519,97 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#8</t>
-        </is>
-      </c>
-      <c r="B18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Isaac Mbele</t>
-        </is>
-      </c>
-      <c r="C18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-22</t>
-        </is>
-      </c>
-      <c r="D18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-26</t>
-        </is>
-      </c>
-      <c r="E18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22 Sep 2026 WhatsApp 08:15: "Mother so like. Aim not well balanced abo</t>
-        </is>
-      </c>
-      <c r="F18" s="4">
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOAN REPAYMENT HISTORY (all payrolls)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loan #</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Employee</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Payroll week</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recorded at</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Result</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scheduled</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deducted</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Balance before</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Balance after</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#1</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Erick Mpho Molefe</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-11 10:12</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deducted</t>
+        </is>
+      </c>
+      <c r="F21" s="4">
         <v>500</v>
       </c>
-      <c r="G18" s="4">
-        <v>250</v>
-      </c>
-      <c r="H18" s="4">
-        <v>0</v>
-      </c>
-      <c r="I18" s="5">
+      <c r="G21" s="4">
         <v>500</v>
       </c>
-      <c r="J18" s="4">
-        <v>0</v>
-      </c>
-      <c r="K18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">weekly</t>
-        </is>
-      </c>
-      <c r="L18" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">active</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOAN REPAYMENT HISTORY (all payrolls)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Loan #</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Employee</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Payroll week</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recorded at</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Result</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Scheduled</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Deducted</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Balance before</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Balance after</t>
-        </is>
+      <c r="H21" s="4">
+        <v>2000</v>
+      </c>
+      <c r="I21" s="4">
+        <v>1500</v>
       </c>
     </row>
     <row r="22">
@@ -14616,12 +14625,12 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
+          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11 10:12</t>
+          <t xml:space="preserve">2026-08-16 13:37</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
@@ -14636,10 +14645,10 @@
         <v>500</v>
       </c>
       <c r="H22" s="4">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="I22" s="4">
-        <v>1500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="23">
@@ -14655,12 +14664,12 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
+          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16 13:37</t>
+          <t xml:space="preserve">2026-09-07 12:01</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -14675,49 +14684,49 @@
         <v>500</v>
       </c>
       <c r="H23" s="4">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="I23" s="4">
-        <v>1000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#1</t>
+          <t xml:space="preserve">#2</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erick Mpho Molefe</t>
+          <t xml:space="preserve">Isaac Mbele</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07 12:01</t>
+          <t xml:space="preserve">2026-08-11 09:42</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">deducted</t>
+          <t xml:space="preserve">deferred</t>
         </is>
       </c>
       <c r="F24" s="4">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G24" s="4">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="I24" s="4">
-        <v>500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="25">
@@ -14733,30 +14742,30 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-08 → 2026-08-14</t>
+          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-11 09:42</t>
+          <t xml:space="preserve">2026-08-16 13:37</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">deferred</t>
+          <t xml:space="preserve">deducted</t>
         </is>
       </c>
       <c r="F25" s="4">
         <v>300</v>
       </c>
       <c r="G25" s="4">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H25" s="4">
         <v>900</v>
       </c>
       <c r="I25" s="4">
-        <v>900</v>
+        <v>600</v>
       </c>
     </row>
     <row r="26">
@@ -14772,12 +14781,12 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
+          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16 13:37</t>
+          <t xml:space="preserve">2026-09-07 12:01</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -14786,22 +14795,22 @@
         </is>
       </c>
       <c r="F26" s="4">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="G26" s="4">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="H26" s="4">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="I26" s="4">
-        <v>600</v>
+        <v>350</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#2</t>
+          <t xml:space="preserve">#3</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -14811,12 +14820,12 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
+          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07 12:01</t>
+          <t xml:space="preserve">2026-08-16 13:37</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
@@ -14825,16 +14834,16 @@
         </is>
       </c>
       <c r="F27" s="4">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="G27" s="4">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="H27" s="4">
         <v>600</v>
       </c>
       <c r="I27" s="4">
-        <v>350</v>
+        <v>400</v>
       </c>
     </row>
     <row r="28">
@@ -14850,12 +14859,12 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-15 → 2026-08-21</t>
+          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-16 13:37</t>
+          <t xml:space="preserve">2026-09-07 12:01</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
@@ -14864,27 +14873,27 @@
         </is>
       </c>
       <c r="F28" s="4">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="G28" s="4">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="H28" s="4">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="I28" s="4">
-        <v>400</v>
+        <v>150</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#3</t>
+          <t xml:space="preserve">#5</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Isaac Mbele</t>
+          <t xml:space="preserve">Daniel Motaung</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -14899,31 +14908,31 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">deducted</t>
+          <t xml:space="preserve">deferred</t>
         </is>
       </c>
       <c r="F29" s="4">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="G29" s="4">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>400</v>
+        <v>3000</v>
       </c>
       <c r="I29" s="4">
-        <v>150</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">#5</t>
+          <t xml:space="preserve">#6</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Daniel Motaung</t>
+          <t xml:space="preserve">Isaac Mbele</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -14942,54 +14951,15 @@
         </is>
       </c>
       <c r="F30" s="4">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="G30" s="4">
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>3000</v>
+        <v>600</v>
       </c>
       <c r="I30" s="4">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#6</t>
-        </is>
-      </c>
-      <c r="B31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Isaac Mbele</t>
-        </is>
-      </c>
-      <c r="C31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-05 → 2026-09-11</t>
-        </is>
-      </c>
-      <c r="D31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07 12:01</t>
-        </is>
-      </c>
-      <c r="E31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deferred</t>
-        </is>
-      </c>
-      <c r="F31" s="4">
-        <v>600</v>
-      </c>
-      <c r="G31" s="4">
-        <v>0</v>
-      </c>
-      <c r="H31" s="4">
-        <v>600</v>
-      </c>
-      <c r="I31" s="4">
         <v>600</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Takavaudza #9821 Sun 20 Sep -> VENUE R684 (owner); Sunday/holiday matrix by place in docs; auditor xlsx refreshed
</commit_message>
<xml_diff>
--- a/docs/BW_Payroll_2026-09-19_to_25_AUDITOR.xlsx
+++ b/docs/BW_Payroll_2026-09-19_to_25_AUDITOR.xlsx
@@ -6656,18 +6656,18 @@
         <f>IF(N80&lt;&gt;"",N80,M80)</f>
       </c>
       <c r="P80" s="4">
-        <v>450</v>
+        <v>684</v>
       </c>
       <c r="Q80" s="7"/>
       <c r="R80" s="5">
         <f>IF(Q80&lt;&gt;"",Q80,IF(N80&lt;&gt;"",IF(M80&gt;0,ROUND(P80*N80/M80,2),0),P80))</f>
       </c>
       <c r="S80" s="9">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="T80" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">OWNER CORRECTION: Owner 24 Sep: Sunday house work 08:00–14:00 = 6 h × R62,50 × 1.2 (Sunday) = 6 h × R75 = R450,00 (was R375 — Sunday ×1.2 had been left off)</t>
+          <t xml:space="preserve">OWNER CORRECTION: Owner 24 Sep: VENUE — installing lights at the House is event/venue work, not garden work. Sunday 08:00–14:00 = 6 h × R95 × 1.2 = 6 h × R114 = R684,00 (paid R375 on 23 Sep at the flat garden rate; corrected to R450 garden+Sunday, then to R684 venue+Sunday on 24 Sep)</t>
         </is>
       </c>
       <c r="U80" s="6"/>

</xml_diff>